<commit_message>
Fix where consolidate ignore most of the data into duckdb. Fix where crosschecking not found most of all data. Add new column Status | System Status | User Status to Audit_Result excel output. Add filter button like excel to Result table. Change download_full_report() to download_excel_report() in crosscheck module.
</commit_message>
<xml_diff>
--- a/templates/Sample-Excel_Report.xlsx
+++ b/templates/Sample-Excel_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TiiTii\Desktop\AuditCore_DEV\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4600ABE0-16A2-4C95-A2D3-432F93D55B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CEF073-4936-4B5F-8919-9AB9939ED31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="801" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,10 +64,10 @@
     <definedName name="__SR2">#REF!</definedName>
     <definedName name="__wb2" hidden="1">{#N/A,#N/A,FALSE,"1998_SK_DB2";#N/A,#N/A,FALSE,"1999_SK_DB2";#N/A,#N/A,FALSE,"2000_SK_DB2";#N/A,#N/A,FALSE,"SK_VE";#N/A,#N/A,FALSE,"1998_CZ_DB2";#N/A,#N/A,FALSE,"1999_CZ_DB2";#N/A,#N/A,FALSE,"2000_CZ_DB2";#N/A,#N/A,FALSE,"CZ_VE";#N/A,#N/A,FALSE,"1998_XX_DB2";#N/A,#N/A,FALSE,"1999_XX_DB2";#N/A,#N/A,FALSE,"2000_XX_DB2";#N/A,#N/A,FALSE,"XX_VE";#N/A,#N/A,FALSE,"SoKo";#N/A,#N/A,FALSE,"SoErg";#N/A,#N/A,FALSE,"Kon"}</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Annex II-IM Non-State Charge'!$A$9:$K$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Annex I-IM State Charge'!$A$8:$I$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Annex IV-EX'!$A$8:$E$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Annex V-Local Sale'!$A$8:$N$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AnnexIII-Local Pur'!$A$8:$AS$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Annex I-IM State Charge'!$A$9:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Annex IV-EX'!$A$9:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Annex V-Local Sale'!$A$9:$N$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AnnexIII-Local Pur'!$A$9:$AT$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Damco!$B$11:$I$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Sale - Aug'!$A$6:$P$50</definedName>
     <definedName name="_Order1" hidden="1">255</definedName>
@@ -223,7 +223,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3716" uniqueCount="1054">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3717" uniqueCount="1055">
   <si>
     <t>USD</t>
   </si>
@@ -3429,6 +3429,9 @@
   </si>
   <si>
     <t>មតិអ្នកប្រើប្រាស់</t>
+  </si>
+  <si>
+    <t>ស្ថានភាពប្រព័ន្ធ</t>
   </si>
 </sst>
 </file>
@@ -3985,7 +3988,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="54">
+  <borders count="53">
     <border>
       <left/>
       <right/>
@@ -4432,17 +4435,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -4719,15 +4711,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="81" fillId="0" borderId="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="49" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="50" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="80" fillId="0" borderId="51" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="48" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="79" fillId="0" borderId="49" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="80" fillId="0" borderId="50" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="80" fillId="0" borderId="0" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="76" fillId="3" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="53" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="82" fillId="0" borderId="52" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="76" fillId="3" borderId="52" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="83" fillId="0" borderId="52" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="51" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="404">
+  <cellXfs count="402">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="168" fontId="19" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
@@ -4974,7 +4966,7 @@
     <xf numFmtId="174" fontId="65" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="67" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="70" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5141,7 +5133,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="168" fontId="19" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5150,19 +5142,19 @@
     <xf numFmtId="49" fontId="17" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="20" fillId="0" borderId="45" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="44" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5171,22 +5163,22 @@
     <xf numFmtId="49" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="0" borderId="47" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="19" fillId="0" borderId="46" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1" applyAlignment="1">
@@ -5462,6 +5454,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="88" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="84" fillId="0" borderId="0" xfId="25" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="84" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="65" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5475,23 +5479,8 @@
     <xf numFmtId="0" fontId="66" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="36" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="65" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="65" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="173" fontId="65" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="67" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5511,10 +5500,20 @@
     <xf numFmtId="0" fontId="67" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="84" fillId="0" borderId="0" xfId="25" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="87" fillId="6" borderId="4" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="84" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="87" fillId="6" borderId="10" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="6" borderId="3" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="0" borderId="0" xfId="25" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="85" fillId="0" borderId="4" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5532,29 +5531,6 @@
     <xf numFmtId="164" fontId="85" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="84" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="85" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="87" fillId="6" borderId="4" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="87" fillId="6" borderId="4" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="87" fillId="6" borderId="10" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="87" fillId="6" borderId="3" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="87" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="86" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="77" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5564,6 +5540,13 @@
     <xf numFmtId="0" fontId="77" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="84" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="6" borderId="4" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="86" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5747,10 +5730,10 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5762,13 +5745,13 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="171" fontId="48" fillId="0" borderId="4" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5833,6 +5816,9 @@
     </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="65" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -8847,41 +8833,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="33.6">
-      <c r="A1" s="377" t="s">
+      <c r="A1" s="374" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="377"/>
-      <c r="C1" s="377"/>
-      <c r="D1" s="377"/>
-      <c r="E1" s="377"/>
-      <c r="F1" s="377"/>
-      <c r="G1" s="377"/>
-      <c r="H1" s="377"/>
-      <c r="I1" s="377"/>
-      <c r="J1" s="378"/>
+      <c r="B1" s="374"/>
+      <c r="C1" s="374"/>
+      <c r="D1" s="374"/>
+      <c r="E1" s="374"/>
+      <c r="F1" s="374"/>
+      <c r="G1" s="374"/>
+      <c r="H1" s="374"/>
+      <c r="I1" s="374"/>
+      <c r="J1" s="375"/>
     </row>
     <row r="2" spans="1:10" ht="33.6">
-      <c r="A2" s="377" t="s">
+      <c r="A2" s="374" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="377"/>
-      <c r="C2" s="377"/>
-      <c r="D2" s="377"/>
-      <c r="E2" s="377"/>
-      <c r="F2" s="377"/>
-      <c r="G2" s="377"/>
-      <c r="H2" s="377"/>
-      <c r="I2" s="377"/>
-      <c r="J2" s="378"/>
+      <c r="B2" s="374"/>
+      <c r="C2" s="374"/>
+      <c r="D2" s="374"/>
+      <c r="E2" s="374"/>
+      <c r="F2" s="374"/>
+      <c r="G2" s="374"/>
+      <c r="H2" s="374"/>
+      <c r="I2" s="374"/>
+      <c r="J2" s="375"/>
     </row>
     <row r="3" spans="1:10" ht="27">
-      <c r="A3" s="379" t="s">
+      <c r="A3" s="376" t="s">
         <v>723</v>
       </c>
-      <c r="B3" s="379"/>
-      <c r="C3" s="379"/>
-      <c r="D3" s="379"/>
-      <c r="E3" s="379"/>
+      <c r="B3" s="376"/>
+      <c r="C3" s="376"/>
+      <c r="D3" s="376"/>
+      <c r="E3" s="376"/>
       <c r="F3" s="159"/>
       <c r="G3" s="159"/>
       <c r="H3" s="159"/>
@@ -8889,12 +8875,12 @@
       <c r="J3" s="160"/>
     </row>
     <row r="4" spans="1:10" ht="27">
-      <c r="A4" s="339" t="s">
+      <c r="A4" s="336" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="339"/>
-      <c r="C4" s="339"/>
-      <c r="D4" s="339"/>
+      <c r="B4" s="336"/>
+      <c r="C4" s="336"/>
+      <c r="D4" s="336"/>
       <c r="E4" s="159"/>
       <c r="F4" s="159"/>
       <c r="G4" s="159"/>
@@ -8903,47 +8889,47 @@
       <c r="J4" s="160"/>
     </row>
     <row r="5" spans="1:10" ht="25.2">
-      <c r="A5" s="359" t="s">
+      <c r="A5" s="356" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="362" t="s">
+      <c r="B5" s="359" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="363"/>
-      <c r="D5" s="364"/>
-      <c r="E5" s="365" t="s">
+      <c r="C5" s="360"/>
+      <c r="D5" s="361"/>
+      <c r="E5" s="362" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="366"/>
-      <c r="G5" s="366"/>
-      <c r="H5" s="366"/>
-      <c r="I5" s="366"/>
-      <c r="J5" s="380" t="s">
+      <c r="F5" s="363"/>
+      <c r="G5" s="363"/>
+      <c r="H5" s="363"/>
+      <c r="I5" s="363"/>
+      <c r="J5" s="377" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="25.2">
-      <c r="A6" s="360"/>
-      <c r="B6" s="370" t="s">
+      <c r="A6" s="357"/>
+      <c r="B6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="371"/>
-      <c r="D6" s="372"/>
-      <c r="E6" s="373" t="s">
+      <c r="C6" s="368"/>
+      <c r="D6" s="369"/>
+      <c r="E6" s="370" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="374" t="s">
+      <c r="F6" s="371" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="370" t="s">
+      <c r="G6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="371"/>
-      <c r="I6" s="372"/>
-      <c r="J6" s="381"/>
+      <c r="H6" s="368"/>
+      <c r="I6" s="369"/>
+      <c r="J6" s="378"/>
     </row>
     <row r="7" spans="1:10" ht="25.2">
-      <c r="A7" s="361"/>
+      <c r="A7" s="358"/>
       <c r="B7" s="155" t="s">
         <v>6</v>
       </c>
@@ -8953,8 +8939,8 @@
       <c r="D7" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="374"/>
-      <c r="F7" s="374"/>
+      <c r="E7" s="371"/>
+      <c r="F7" s="371"/>
       <c r="G7" s="155" t="s">
         <v>6</v>
       </c>
@@ -8964,7 +8950,7 @@
       <c r="I7" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="382"/>
+      <c r="J7" s="379"/>
     </row>
     <row r="8" spans="1:10" ht="18" customHeight="1">
       <c r="A8" s="131">
@@ -22497,10 +22483,10 @@
       <c r="J458" s="161"/>
     </row>
     <row r="459" spans="1:10" ht="24">
-      <c r="A459" s="375" t="s">
+      <c r="A459" s="372" t="s">
         <v>724</v>
       </c>
-      <c r="B459" s="376"/>
+      <c r="B459" s="373"/>
       <c r="C459" s="164"/>
       <c r="D459" s="165">
         <f>SUM(D8:D458)</f>
@@ -22559,41 +22545,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="33.6">
-      <c r="A1" s="377" t="s">
+      <c r="A1" s="374" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="377"/>
-      <c r="C1" s="377"/>
-      <c r="D1" s="377"/>
-      <c r="E1" s="377"/>
-      <c r="F1" s="377"/>
-      <c r="G1" s="377"/>
-      <c r="H1" s="377"/>
-      <c r="I1" s="377"/>
-      <c r="J1" s="378"/>
+      <c r="B1" s="374"/>
+      <c r="C1" s="374"/>
+      <c r="D1" s="374"/>
+      <c r="E1" s="374"/>
+      <c r="F1" s="374"/>
+      <c r="G1" s="374"/>
+      <c r="H1" s="374"/>
+      <c r="I1" s="374"/>
+      <c r="J1" s="375"/>
     </row>
     <row r="2" spans="1:10" ht="33.6">
-      <c r="A2" s="377" t="s">
+      <c r="A2" s="374" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="377"/>
-      <c r="C2" s="377"/>
-      <c r="D2" s="377"/>
-      <c r="E2" s="377"/>
-      <c r="F2" s="377"/>
-      <c r="G2" s="377"/>
-      <c r="H2" s="377"/>
-      <c r="I2" s="377"/>
-      <c r="J2" s="378"/>
+      <c r="B2" s="374"/>
+      <c r="C2" s="374"/>
+      <c r="D2" s="374"/>
+      <c r="E2" s="374"/>
+      <c r="F2" s="374"/>
+      <c r="G2" s="374"/>
+      <c r="H2" s="374"/>
+      <c r="I2" s="374"/>
+      <c r="J2" s="375"/>
     </row>
     <row r="3" spans="1:10" ht="27">
-      <c r="A3" s="379" t="s">
+      <c r="A3" s="376" t="s">
         <v>723</v>
       </c>
-      <c r="B3" s="379"/>
-      <c r="C3" s="379"/>
-      <c r="D3" s="379"/>
-      <c r="E3" s="379"/>
+      <c r="B3" s="376"/>
+      <c r="C3" s="376"/>
+      <c r="D3" s="376"/>
+      <c r="E3" s="376"/>
       <c r="F3" s="159"/>
       <c r="G3" s="159"/>
       <c r="H3" s="159"/>
@@ -22601,12 +22587,12 @@
       <c r="J3" s="160"/>
     </row>
     <row r="4" spans="1:10" ht="27">
-      <c r="A4" s="339" t="s">
+      <c r="A4" s="336" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="339"/>
-      <c r="C4" s="339"/>
-      <c r="D4" s="339"/>
+      <c r="B4" s="336"/>
+      <c r="C4" s="336"/>
+      <c r="D4" s="336"/>
       <c r="E4" s="159"/>
       <c r="F4" s="159"/>
       <c r="G4" s="159"/>
@@ -22615,47 +22601,47 @@
       <c r="J4" s="160"/>
     </row>
     <row r="5" spans="1:10" ht="25.2">
-      <c r="A5" s="359" t="s">
+      <c r="A5" s="356" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="362" t="s">
+      <c r="B5" s="359" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="363"/>
-      <c r="D5" s="364"/>
-      <c r="E5" s="365" t="s">
+      <c r="C5" s="360"/>
+      <c r="D5" s="361"/>
+      <c r="E5" s="362" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="366"/>
-      <c r="G5" s="366"/>
-      <c r="H5" s="366"/>
-      <c r="I5" s="366"/>
-      <c r="J5" s="380" t="s">
+      <c r="F5" s="363"/>
+      <c r="G5" s="363"/>
+      <c r="H5" s="363"/>
+      <c r="I5" s="363"/>
+      <c r="J5" s="377" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="25.2">
-      <c r="A6" s="360"/>
-      <c r="B6" s="370" t="s">
+      <c r="A6" s="357"/>
+      <c r="B6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="371"/>
-      <c r="D6" s="372"/>
-      <c r="E6" s="373" t="s">
+      <c r="C6" s="368"/>
+      <c r="D6" s="369"/>
+      <c r="E6" s="370" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="374" t="s">
+      <c r="F6" s="371" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="370" t="s">
+      <c r="G6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="371"/>
-      <c r="I6" s="372"/>
-      <c r="J6" s="381"/>
+      <c r="H6" s="368"/>
+      <c r="I6" s="369"/>
+      <c r="J6" s="378"/>
     </row>
     <row r="7" spans="1:10" ht="25.2">
-      <c r="A7" s="361"/>
+      <c r="A7" s="358"/>
       <c r="B7" s="155" t="s">
         <v>6</v>
       </c>
@@ -22665,8 +22651,8 @@
       <c r="D7" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="374"/>
-      <c r="F7" s="374"/>
+      <c r="E7" s="371"/>
+      <c r="F7" s="371"/>
       <c r="G7" s="155" t="s">
         <v>6</v>
       </c>
@@ -22676,7 +22662,7 @@
       <c r="I7" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="382"/>
+      <c r="J7" s="379"/>
     </row>
     <row r="8" spans="1:10" ht="25.2">
       <c r="A8" s="169"/>
@@ -23093,39 +23079,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="178" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A1" s="388" t="s">
+      <c r="A1" s="385" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="388"/>
-      <c r="C1" s="388"/>
-      <c r="D1" s="388"/>
-      <c r="E1" s="388"/>
-      <c r="F1" s="388"/>
-      <c r="G1" s="388"/>
-      <c r="H1" s="388"/>
-      <c r="I1" s="388"/>
-      <c r="J1" s="388"/>
-      <c r="K1" s="388"/>
-      <c r="L1" s="388"/>
-      <c r="M1" s="388"/>
+      <c r="B1" s="385"/>
+      <c r="C1" s="385"/>
+      <c r="D1" s="385"/>
+      <c r="E1" s="385"/>
+      <c r="F1" s="385"/>
+      <c r="G1" s="385"/>
+      <c r="H1" s="385"/>
+      <c r="I1" s="385"/>
+      <c r="J1" s="385"/>
+      <c r="K1" s="385"/>
+      <c r="L1" s="385"/>
+      <c r="M1" s="385"/>
       <c r="N1" s="177"/>
     </row>
     <row r="2" spans="1:15" s="179" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A2" s="389" t="s">
+      <c r="A2" s="386" t="s">
         <v>907</v>
       </c>
-      <c r="B2" s="389"/>
-      <c r="C2" s="389"/>
-      <c r="D2" s="389"/>
-      <c r="E2" s="389"/>
-      <c r="F2" s="389"/>
-      <c r="G2" s="389"/>
-      <c r="H2" s="389"/>
-      <c r="I2" s="389"/>
-      <c r="J2" s="389"/>
-      <c r="K2" s="389"/>
-      <c r="L2" s="389"/>
-      <c r="M2" s="389"/>
+      <c r="B2" s="386"/>
+      <c r="C2" s="386"/>
+      <c r="D2" s="386"/>
+      <c r="E2" s="386"/>
+      <c r="F2" s="386"/>
+      <c r="G2" s="386"/>
+      <c r="H2" s="386"/>
+      <c r="I2" s="386"/>
+      <c r="J2" s="386"/>
+      <c r="K2" s="386"/>
+      <c r="L2" s="386"/>
+      <c r="M2" s="386"/>
       <c r="N2" s="177"/>
     </row>
     <row r="3" spans="1:15" s="189" customFormat="1" ht="22.5" customHeight="1">
@@ -23173,22 +23159,22 @@
       <c r="O4" s="188"/>
     </row>
     <row r="5" spans="1:15" s="198" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A5" s="390" t="s">
+      <c r="A5" s="387" t="s">
         <v>755</v>
       </c>
-      <c r="B5" s="391"/>
-      <c r="C5" s="391"/>
-      <c r="D5" s="391"/>
-      <c r="E5" s="391"/>
-      <c r="F5" s="391"/>
-      <c r="G5" s="391"/>
-      <c r="H5" s="391"/>
-      <c r="I5" s="392" t="s">
+      <c r="B5" s="388"/>
+      <c r="C5" s="388"/>
+      <c r="D5" s="388"/>
+      <c r="E5" s="388"/>
+      <c r="F5" s="388"/>
+      <c r="G5" s="388"/>
+      <c r="H5" s="388"/>
+      <c r="I5" s="389" t="s">
         <v>756</v>
       </c>
-      <c r="J5" s="392"/>
-      <c r="K5" s="392"/>
-      <c r="L5" s="392"/>
+      <c r="J5" s="389"/>
+      <c r="K5" s="389"/>
+      <c r="L5" s="389"/>
       <c r="M5" s="199"/>
     </row>
     <row r="6" spans="1:15" s="198" customFormat="1" ht="14.25" customHeight="1">
@@ -23207,17 +23193,17 @@
       <c r="E6" s="201" t="s">
         <v>760</v>
       </c>
-      <c r="F6" s="393" t="s">
+      <c r="F6" s="390" t="s">
         <v>761</v>
       </c>
-      <c r="G6" s="393"/>
+      <c r="G6" s="390"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="394" t="s">
+      <c r="I6" s="391" t="s">
         <v>762</v>
       </c>
-      <c r="J6" s="395"/>
-      <c r="K6" s="395"/>
-      <c r="L6" s="395"/>
+      <c r="J6" s="392"/>
+      <c r="K6" s="392"/>
+      <c r="L6" s="392"/>
       <c r="M6" s="202" t="s">
         <v>763</v>
       </c>
@@ -23237,14 +23223,14 @@
       <c r="H7" s="207" t="s">
         <v>765</v>
       </c>
-      <c r="I7" s="399" t="s">
+      <c r="I7" s="396" t="s">
         <v>766</v>
       </c>
-      <c r="J7" s="399"/>
-      <c r="K7" s="399" t="s">
+      <c r="J7" s="396"/>
+      <c r="K7" s="396" t="s">
         <v>767</v>
       </c>
-      <c r="L7" s="399"/>
+      <c r="L7" s="396"/>
       <c r="M7" s="202" t="s">
         <v>768</v>
       </c>
@@ -23697,13 +23683,13 @@
       </c>
     </row>
     <row r="23" spans="1:14" s="224" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A23" s="383">
+      <c r="A23" s="380">
         <f>L4</f>
         <v>4088</v>
       </c>
-      <c r="B23" s="383"/>
-      <c r="C23" s="383"/>
-      <c r="D23" s="383"/>
+      <c r="B23" s="380"/>
+      <c r="C23" s="380"/>
+      <c r="D23" s="380"/>
       <c r="E23" s="222" t="s">
         <v>847</v>
       </c>
@@ -23726,12 +23712,12 @@
       </c>
     </row>
     <row r="24" spans="1:14" s="224" customFormat="1" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A24" s="384" t="s">
+      <c r="A24" s="381" t="s">
         <v>848</v>
       </c>
-      <c r="B24" s="385"/>
-      <c r="C24" s="385"/>
-      <c r="D24" s="385"/>
+      <c r="B24" s="382"/>
+      <c r="C24" s="382"/>
+      <c r="D24" s="382"/>
       <c r="E24" s="225" t="s">
         <v>0</v>
       </c>
@@ -23800,22 +23786,22 @@
       <c r="E26" s="230"/>
       <c r="F26" s="19"/>
       <c r="G26" s="230"/>
-      <c r="H26" s="386" t="s">
+      <c r="H26" s="383" t="s">
         <v>853</v>
       </c>
-      <c r="I26" s="386"/>
-      <c r="J26" s="386"/>
-      <c r="K26" s="386"/>
-      <c r="L26" s="386"/>
-      <c r="M26" s="386"/>
+      <c r="I26" s="383"/>
+      <c r="J26" s="383"/>
+      <c r="K26" s="383"/>
+      <c r="L26" s="383"/>
+      <c r="M26" s="383"/>
     </row>
     <row r="27" spans="1:14" ht="19.5" customHeight="1">
-      <c r="H27" s="387"/>
-      <c r="I27" s="387"/>
-      <c r="J27" s="387"/>
-      <c r="K27" s="387"/>
-      <c r="L27" s="387"/>
-      <c r="M27" s="387"/>
+      <c r="H27" s="384"/>
+      <c r="I27" s="384"/>
+      <c r="J27" s="384"/>
+      <c r="K27" s="384"/>
+      <c r="L27" s="384"/>
+      <c r="M27" s="384"/>
       <c r="N27" s="21">
         <f>H23*1%</f>
         <v>18908527.420000002</v>
@@ -23836,9 +23822,9 @@
         <v>953</v>
       </c>
       <c r="H29" s="236"/>
-      <c r="I29" s="396"/>
-      <c r="J29" s="396"/>
-      <c r="K29" s="396"/>
+      <c r="I29" s="393"/>
+      <c r="J29" s="393"/>
+      <c r="K29" s="393"/>
       <c r="L29" s="236"/>
     </row>
     <row r="30" spans="1:14" ht="14.25" customHeight="1">
@@ -23917,18 +23903,18 @@
       <c r="K35" s="224"/>
     </row>
     <row r="36" spans="6:13" ht="14.25" customHeight="1">
-      <c r="H36" s="397"/>
-      <c r="I36" s="397"/>
+      <c r="H36" s="394"/>
+      <c r="I36" s="394"/>
       <c r="J36" s="224"/>
       <c r="K36" s="224"/>
       <c r="M36" s="242"/>
     </row>
     <row r="37" spans="6:13" ht="14.25" hidden="1" customHeight="1">
-      <c r="H37" s="398">
+      <c r="H37" s="395">
         <f>H24*1%</f>
         <v>4625.3736350293548</v>
       </c>
-      <c r="I37" s="398"/>
+      <c r="I37" s="395"/>
     </row>
     <row r="38" spans="6:13" ht="14.25" customHeight="1">
       <c r="H38" s="29"/>
@@ -24012,39 +23998,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="178" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A1" s="388" t="s">
+      <c r="A1" s="385" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="388"/>
-      <c r="C1" s="388"/>
-      <c r="D1" s="388"/>
-      <c r="E1" s="388"/>
-      <c r="F1" s="388"/>
-      <c r="G1" s="388"/>
-      <c r="H1" s="388"/>
-      <c r="I1" s="388"/>
-      <c r="J1" s="388"/>
-      <c r="K1" s="388"/>
-      <c r="L1" s="388"/>
-      <c r="M1" s="388"/>
+      <c r="B1" s="385"/>
+      <c r="C1" s="385"/>
+      <c r="D1" s="385"/>
+      <c r="E1" s="385"/>
+      <c r="F1" s="385"/>
+      <c r="G1" s="385"/>
+      <c r="H1" s="385"/>
+      <c r="I1" s="385"/>
+      <c r="J1" s="385"/>
+      <c r="K1" s="385"/>
+      <c r="L1" s="385"/>
+      <c r="M1" s="385"/>
       <c r="N1" s="177"/>
     </row>
     <row r="2" spans="1:15" s="179" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A2" s="389" t="s">
+      <c r="A2" s="386" t="s">
         <v>854</v>
       </c>
-      <c r="B2" s="389"/>
-      <c r="C2" s="389"/>
-      <c r="D2" s="389"/>
-      <c r="E2" s="389"/>
-      <c r="F2" s="389"/>
-      <c r="G2" s="389"/>
-      <c r="H2" s="389"/>
-      <c r="I2" s="389"/>
-      <c r="J2" s="389"/>
-      <c r="K2" s="389"/>
-      <c r="L2" s="389"/>
-      <c r="M2" s="389"/>
+      <c r="B2" s="386"/>
+      <c r="C2" s="386"/>
+      <c r="D2" s="386"/>
+      <c r="E2" s="386"/>
+      <c r="F2" s="386"/>
+      <c r="G2" s="386"/>
+      <c r="H2" s="386"/>
+      <c r="I2" s="386"/>
+      <c r="J2" s="386"/>
+      <c r="K2" s="386"/>
+      <c r="L2" s="386"/>
+      <c r="M2" s="386"/>
       <c r="N2" s="177"/>
     </row>
     <row r="3" spans="1:15" s="189" customFormat="1" ht="22.5" customHeight="1">
@@ -24092,22 +24078,22 @@
       <c r="O4" s="188"/>
     </row>
     <row r="5" spans="1:15" s="198" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A5" s="390" t="s">
+      <c r="A5" s="387" t="s">
         <v>755</v>
       </c>
-      <c r="B5" s="391"/>
-      <c r="C5" s="391"/>
-      <c r="D5" s="391"/>
-      <c r="E5" s="391"/>
-      <c r="F5" s="391"/>
-      <c r="G5" s="391"/>
-      <c r="H5" s="391"/>
-      <c r="I5" s="392" t="s">
+      <c r="B5" s="388"/>
+      <c r="C5" s="388"/>
+      <c r="D5" s="388"/>
+      <c r="E5" s="388"/>
+      <c r="F5" s="388"/>
+      <c r="G5" s="388"/>
+      <c r="H5" s="388"/>
+      <c r="I5" s="389" t="s">
         <v>756</v>
       </c>
-      <c r="J5" s="392"/>
-      <c r="K5" s="392"/>
-      <c r="L5" s="392"/>
+      <c r="J5" s="389"/>
+      <c r="K5" s="389"/>
+      <c r="L5" s="389"/>
       <c r="M5" s="199"/>
     </row>
     <row r="6" spans="1:15" s="198" customFormat="1" ht="14.25" customHeight="1">
@@ -24126,17 +24112,17 @@
       <c r="E6" s="201" t="s">
         <v>760</v>
       </c>
-      <c r="F6" s="393" t="s">
+      <c r="F6" s="390" t="s">
         <v>761</v>
       </c>
-      <c r="G6" s="393"/>
+      <c r="G6" s="390"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="394" t="s">
+      <c r="I6" s="391" t="s">
         <v>762</v>
       </c>
-      <c r="J6" s="395"/>
-      <c r="K6" s="395"/>
-      <c r="L6" s="395"/>
+      <c r="J6" s="392"/>
+      <c r="K6" s="392"/>
+      <c r="L6" s="392"/>
       <c r="M6" s="202" t="s">
         <v>763</v>
       </c>
@@ -24156,14 +24142,14 @@
       <c r="H7" s="207" t="s">
         <v>765</v>
       </c>
-      <c r="I7" s="399" t="s">
+      <c r="I7" s="396" t="s">
         <v>766</v>
       </c>
-      <c r="J7" s="399"/>
-      <c r="K7" s="399" t="s">
+      <c r="J7" s="396"/>
+      <c r="K7" s="396" t="s">
         <v>767</v>
       </c>
-      <c r="L7" s="399"/>
+      <c r="L7" s="396"/>
       <c r="M7" s="202" t="s">
         <v>768</v>
       </c>
@@ -24826,13 +24812,13 @@
       </c>
     </row>
     <row r="30" spans="1:13" s="224" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A30" s="383">
+      <c r="A30" s="380">
         <f>L4</f>
         <v>4099</v>
       </c>
-      <c r="B30" s="383"/>
-      <c r="C30" s="383"/>
-      <c r="D30" s="383"/>
+      <c r="B30" s="380"/>
+      <c r="C30" s="380"/>
+      <c r="D30" s="380"/>
       <c r="E30" s="222" t="s">
         <v>847</v>
       </c>
@@ -24855,12 +24841,12 @@
       </c>
     </row>
     <row r="31" spans="1:13" s="224" customFormat="1" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A31" s="384" t="s">
+      <c r="A31" s="381" t="s">
         <v>848</v>
       </c>
-      <c r="B31" s="385"/>
-      <c r="C31" s="385"/>
-      <c r="D31" s="385"/>
+      <c r="B31" s="382"/>
+      <c r="C31" s="382"/>
+      <c r="D31" s="382"/>
       <c r="E31" s="225" t="s">
         <v>0</v>
       </c>
@@ -24929,22 +24915,22 @@
       <c r="E33" s="230"/>
       <c r="F33" s="19"/>
       <c r="G33" s="230"/>
-      <c r="H33" s="386" t="s">
+      <c r="H33" s="383" t="s">
         <v>853</v>
       </c>
-      <c r="I33" s="386"/>
-      <c r="J33" s="386"/>
-      <c r="K33" s="386"/>
-      <c r="L33" s="386"/>
-      <c r="M33" s="386"/>
+      <c r="I33" s="383"/>
+      <c r="J33" s="383"/>
+      <c r="K33" s="383"/>
+      <c r="L33" s="383"/>
+      <c r="M33" s="383"/>
     </row>
     <row r="34" spans="1:14" ht="19.5" customHeight="1">
-      <c r="H34" s="387"/>
-      <c r="I34" s="387"/>
-      <c r="J34" s="387"/>
-      <c r="K34" s="387"/>
-      <c r="L34" s="387"/>
-      <c r="M34" s="387"/>
+      <c r="H34" s="384"/>
+      <c r="I34" s="384"/>
+      <c r="J34" s="384"/>
+      <c r="K34" s="384"/>
+      <c r="L34" s="384"/>
+      <c r="M34" s="384"/>
       <c r="N34" s="21"/>
     </row>
     <row r="35" spans="1:14" ht="18" hidden="1" customHeight="1">
@@ -24959,9 +24945,9 @@
     </row>
     <row r="36" spans="1:14" ht="14.25" customHeight="1">
       <c r="H36" s="236"/>
-      <c r="I36" s="396"/>
-      <c r="J36" s="396"/>
-      <c r="K36" s="396"/>
+      <c r="I36" s="393"/>
+      <c r="J36" s="393"/>
+      <c r="K36" s="393"/>
       <c r="L36" s="236"/>
     </row>
     <row r="37" spans="1:14" ht="14.25" customHeight="1">
@@ -24972,8 +24958,8 @@
     </row>
     <row r="38" spans="1:14" ht="14.25" customHeight="1">
       <c r="F38" s="26"/>
-      <c r="G38" s="400"/>
-      <c r="H38" s="400"/>
+      <c r="G38" s="397"/>
+      <c r="H38" s="397"/>
       <c r="I38" s="243"/>
     </row>
     <row r="39" spans="1:14" ht="14.25" customHeight="1">
@@ -25007,18 +24993,18 @@
       <c r="K42" s="224"/>
     </row>
     <row r="43" spans="1:14" ht="14.25" customHeight="1">
-      <c r="H43" s="397"/>
-      <c r="I43" s="397"/>
+      <c r="H43" s="394"/>
+      <c r="I43" s="394"/>
       <c r="J43" s="224"/>
       <c r="K43" s="224"/>
       <c r="M43" s="242"/>
     </row>
     <row r="44" spans="1:14" ht="14.25" hidden="1" customHeight="1">
-      <c r="H44" s="398">
+      <c r="H44" s="395">
         <f>H31*1%</f>
         <v>8245.1327201756521</v>
       </c>
-      <c r="I44" s="398"/>
+      <c r="I44" s="395"/>
     </row>
     <row r="45" spans="1:14" ht="14.25" customHeight="1">
       <c r="H45" s="29"/>
@@ -25104,41 +25090,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="178" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A1" s="388" t="s">
+      <c r="A1" s="385" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="388"/>
-      <c r="C1" s="388"/>
-      <c r="D1" s="388"/>
-      <c r="E1" s="388"/>
-      <c r="F1" s="388"/>
-      <c r="G1" s="388"/>
-      <c r="H1" s="388"/>
-      <c r="I1" s="388"/>
-      <c r="J1" s="388"/>
-      <c r="K1" s="388"/>
-      <c r="L1" s="388"/>
-      <c r="M1" s="388"/>
-      <c r="N1" s="388"/>
+      <c r="B1" s="385"/>
+      <c r="C1" s="385"/>
+      <c r="D1" s="385"/>
+      <c r="E1" s="385"/>
+      <c r="F1" s="385"/>
+      <c r="G1" s="385"/>
+      <c r="H1" s="385"/>
+      <c r="I1" s="385"/>
+      <c r="J1" s="385"/>
+      <c r="K1" s="385"/>
+      <c r="L1" s="385"/>
+      <c r="M1" s="385"/>
+      <c r="N1" s="385"/>
       <c r="O1" s="177"/>
     </row>
     <row r="2" spans="1:16" s="179" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A2" s="389" t="s">
+      <c r="A2" s="386" t="s">
         <v>750</v>
       </c>
-      <c r="B2" s="389"/>
-      <c r="C2" s="389"/>
-      <c r="D2" s="389"/>
-      <c r="E2" s="389"/>
-      <c r="F2" s="389"/>
-      <c r="G2" s="389"/>
-      <c r="H2" s="389"/>
-      <c r="I2" s="389"/>
-      <c r="J2" s="389"/>
-      <c r="K2" s="389"/>
-      <c r="L2" s="389"/>
-      <c r="M2" s="389"/>
-      <c r="N2" s="389"/>
+      <c r="B2" s="386"/>
+      <c r="C2" s="386"/>
+      <c r="D2" s="386"/>
+      <c r="E2" s="386"/>
+      <c r="F2" s="386"/>
+      <c r="G2" s="386"/>
+      <c r="H2" s="386"/>
+      <c r="I2" s="386"/>
+      <c r="J2" s="386"/>
+      <c r="K2" s="386"/>
+      <c r="L2" s="386"/>
+      <c r="M2" s="386"/>
+      <c r="N2" s="386"/>
       <c r="O2" s="177"/>
     </row>
     <row r="3" spans="1:16" s="189" customFormat="1" ht="22.5" customHeight="1">
@@ -25188,23 +25174,23 @@
       <c r="P4" s="188"/>
     </row>
     <row r="5" spans="1:16" s="198" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A5" s="390" t="s">
+      <c r="A5" s="387" t="s">
         <v>755</v>
       </c>
-      <c r="B5" s="391"/>
-      <c r="C5" s="391"/>
-      <c r="D5" s="391"/>
-      <c r="E5" s="391"/>
-      <c r="F5" s="391"/>
-      <c r="G5" s="391"/>
-      <c r="H5" s="391"/>
-      <c r="I5" s="391"/>
-      <c r="J5" s="392" t="s">
+      <c r="B5" s="388"/>
+      <c r="C5" s="388"/>
+      <c r="D5" s="388"/>
+      <c r="E5" s="388"/>
+      <c r="F5" s="388"/>
+      <c r="G5" s="388"/>
+      <c r="H5" s="388"/>
+      <c r="I5" s="388"/>
+      <c r="J5" s="389" t="s">
         <v>756</v>
       </c>
-      <c r="K5" s="392"/>
-      <c r="L5" s="392"/>
-      <c r="M5" s="392"/>
+      <c r="K5" s="389"/>
+      <c r="L5" s="389"/>
+      <c r="M5" s="389"/>
       <c r="N5" s="199"/>
     </row>
     <row r="6" spans="1:16" s="198" customFormat="1" ht="14.25" customHeight="1">
@@ -25223,18 +25209,18 @@
       <c r="E6" s="201" t="s">
         <v>760</v>
       </c>
-      <c r="F6" s="393" t="s">
+      <c r="F6" s="390" t="s">
         <v>761</v>
       </c>
-      <c r="G6" s="393"/>
-      <c r="H6" s="393"/>
+      <c r="G6" s="390"/>
+      <c r="H6" s="390"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="394" t="s">
+      <c r="J6" s="391" t="s">
         <v>762</v>
       </c>
-      <c r="K6" s="395"/>
-      <c r="L6" s="395"/>
-      <c r="M6" s="395"/>
+      <c r="K6" s="392"/>
+      <c r="L6" s="392"/>
+      <c r="M6" s="392"/>
       <c r="N6" s="202" t="s">
         <v>763</v>
       </c>
@@ -25247,22 +25233,22 @@
         <v>764</v>
       </c>
       <c r="E7" s="206"/>
-      <c r="F7" s="401" t="s">
+      <c r="F7" s="398" t="s">
         <v>756</v>
       </c>
-      <c r="G7" s="402"/>
-      <c r="H7" s="403"/>
+      <c r="G7" s="399"/>
+      <c r="H7" s="400"/>
       <c r="I7" s="207" t="s">
         <v>765</v>
       </c>
-      <c r="J7" s="399" t="s">
+      <c r="J7" s="396" t="s">
         <v>766</v>
       </c>
-      <c r="K7" s="399"/>
-      <c r="L7" s="399" t="s">
+      <c r="K7" s="396"/>
+      <c r="L7" s="396" t="s">
         <v>767</v>
       </c>
-      <c r="M7" s="399"/>
+      <c r="M7" s="396"/>
       <c r="N7" s="202" t="s">
         <v>768</v>
       </c>
@@ -25273,11 +25259,11 @@
       <c r="C8" s="209"/>
       <c r="D8" s="210"/>
       <c r="E8" s="211"/>
-      <c r="F8" s="401" t="s">
+      <c r="F8" s="398" t="s">
         <v>769</v>
       </c>
-      <c r="G8" s="402"/>
-      <c r="H8" s="403"/>
+      <c r="G8" s="399"/>
+      <c r="H8" s="400"/>
       <c r="I8" s="213" t="s">
         <v>770</v>
       </c>
@@ -26551,13 +26537,13 @@
       </c>
     </row>
     <row r="47" spans="1:14" s="224" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A47" s="383">
+      <c r="A47" s="380">
         <f>M4</f>
         <v>4095</v>
       </c>
-      <c r="B47" s="383"/>
-      <c r="C47" s="383"/>
-      <c r="D47" s="383"/>
+      <c r="B47" s="380"/>
+      <c r="C47" s="380"/>
+      <c r="D47" s="380"/>
       <c r="E47" s="222" t="s">
         <v>847</v>
       </c>
@@ -26578,12 +26564,12 @@
       </c>
     </row>
     <row r="48" spans="1:14" s="224" customFormat="1" ht="14.25" customHeight="1" thickBot="1">
-      <c r="A48" s="384" t="s">
+      <c r="A48" s="381" t="s">
         <v>848</v>
       </c>
-      <c r="B48" s="385"/>
-      <c r="C48" s="385"/>
-      <c r="D48" s="385"/>
+      <c r="B48" s="382"/>
+      <c r="C48" s="382"/>
+      <c r="D48" s="382"/>
       <c r="E48" s="225" t="s">
         <v>0</v>
       </c>
@@ -26655,22 +26641,22 @@
       <c r="F50" s="19"/>
       <c r="G50" s="19"/>
       <c r="H50" s="230"/>
-      <c r="I50" s="386" t="s">
+      <c r="I50" s="383" t="s">
         <v>853</v>
       </c>
-      <c r="J50" s="386"/>
-      <c r="K50" s="386"/>
-      <c r="L50" s="386"/>
-      <c r="M50" s="386"/>
-      <c r="N50" s="386"/>
+      <c r="J50" s="383"/>
+      <c r="K50" s="383"/>
+      <c r="L50" s="383"/>
+      <c r="M50" s="383"/>
+      <c r="N50" s="383"/>
     </row>
     <row r="51" spans="1:15" ht="19.5" customHeight="1">
-      <c r="I51" s="387"/>
-      <c r="J51" s="387"/>
-      <c r="K51" s="387"/>
-      <c r="L51" s="387"/>
-      <c r="M51" s="387"/>
-      <c r="N51" s="387"/>
+      <c r="I51" s="384"/>
+      <c r="J51" s="384"/>
+      <c r="K51" s="384"/>
+      <c r="L51" s="384"/>
+      <c r="M51" s="384"/>
+      <c r="N51" s="384"/>
       <c r="O51" s="21"/>
     </row>
     <row r="52" spans="1:15" ht="18" hidden="1" customHeight="1">
@@ -26685,9 +26671,9 @@
     </row>
     <row r="53" spans="1:15" ht="14.25" customHeight="1">
       <c r="I53" s="236"/>
-      <c r="J53" s="396"/>
-      <c r="K53" s="396"/>
-      <c r="L53" s="396"/>
+      <c r="J53" s="393"/>
+      <c r="K53" s="393"/>
+      <c r="L53" s="393"/>
       <c r="M53" s="236"/>
     </row>
     <row r="54" spans="1:15" ht="14.25" customHeight="1">
@@ -26700,8 +26686,8 @@
     <row r="55" spans="1:15" ht="14.25" customHeight="1">
       <c r="F55" s="26"/>
       <c r="G55" s="26"/>
-      <c r="H55" s="400"/>
-      <c r="I55" s="400"/>
+      <c r="H55" s="397"/>
+      <c r="I55" s="397"/>
       <c r="J55" s="243"/>
     </row>
     <row r="56" spans="1:15" ht="14.25" customHeight="1">
@@ -26738,18 +26724,18 @@
       <c r="L59" s="224"/>
     </row>
     <row r="60" spans="1:15" ht="14.25" customHeight="1">
-      <c r="I60" s="397"/>
-      <c r="J60" s="397"/>
+      <c r="I60" s="394"/>
+      <c r="J60" s="394"/>
       <c r="K60" s="224"/>
       <c r="L60" s="224"/>
       <c r="N60" s="242"/>
     </row>
     <row r="61" spans="1:15" ht="14.25" hidden="1" customHeight="1">
-      <c r="I61" s="398">
+      <c r="I61" s="395">
         <f>I48*1%</f>
         <v>12759.654327228329</v>
       </c>
-      <c r="J61" s="398"/>
+      <c r="J61" s="395"/>
     </row>
     <row r="62" spans="1:15" ht="14.25" customHeight="1">
       <c r="I62" s="29"/>
@@ -26831,40 +26817,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="60" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="278" t="s">
+      <c r="A1" s="282" t="s">
         <v>966</v>
       </c>
-      <c r="B1" s="278"/>
-      <c r="C1" s="278"/>
-      <c r="D1" s="278"/>
-      <c r="E1" s="278"/>
-      <c r="F1" s="278"/>
-      <c r="G1" s="278"/>
-      <c r="H1" s="278"/>
+      <c r="B1" s="282"/>
+      <c r="C1" s="282"/>
+      <c r="D1" s="282"/>
+      <c r="E1" s="282"/>
+      <c r="F1" s="282"/>
+      <c r="G1" s="282"/>
+      <c r="H1" s="282"/>
     </row>
     <row r="2" spans="1:9" s="60" customFormat="1" ht="30" customHeight="1">
-      <c r="A2" s="278" t="s">
+      <c r="A2" s="282" t="s">
         <v>989</v>
       </c>
-      <c r="B2" s="278"/>
-      <c r="C2" s="278"/>
-      <c r="D2" s="278"/>
-      <c r="E2" s="278"/>
-      <c r="F2" s="278"/>
-      <c r="G2" s="278"/>
-      <c r="H2" s="278"/>
+      <c r="B2" s="282"/>
+      <c r="C2" s="282"/>
+      <c r="D2" s="282"/>
+      <c r="E2" s="282"/>
+      <c r="F2" s="282"/>
+      <c r="G2" s="282"/>
+      <c r="H2" s="282"/>
     </row>
     <row r="3" spans="1:9" s="60" customFormat="1" ht="30" customHeight="1">
-      <c r="A3" s="278" t="s">
+      <c r="A3" s="282" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="278"/>
-      <c r="C3" s="278"/>
-      <c r="D3" s="278"/>
-      <c r="E3" s="278"/>
-      <c r="F3" s="278"/>
-      <c r="G3" s="278"/>
-      <c r="H3" s="278"/>
+      <c r="B3" s="282"/>
+      <c r="C3" s="282"/>
+      <c r="D3" s="282"/>
+      <c r="E3" s="282"/>
+      <c r="F3" s="282"/>
+      <c r="G3" s="282"/>
+      <c r="H3" s="282"/>
     </row>
     <row r="4" spans="1:9" s="60" customFormat="1" ht="30" customHeight="1">
       <c r="A4" s="65" t="s">
@@ -26922,30 +26908,30 @@
       </c>
     </row>
     <row r="7" spans="1:9" s="59" customFormat="1" ht="30" customHeight="1">
-      <c r="A7" s="279" t="s">
+      <c r="A7" s="283" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="279" t="s">
+      <c r="B7" s="283" t="s">
         <v>760</v>
       </c>
-      <c r="C7" s="279" t="s">
+      <c r="C7" s="283" t="s">
         <v>993</v>
       </c>
-      <c r="D7" s="279"/>
-      <c r="E7" s="279" t="s">
+      <c r="D7" s="283"/>
+      <c r="E7" s="283" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="279"/>
-      <c r="G7" s="279" t="s">
+      <c r="F7" s="283"/>
+      <c r="G7" s="283" t="s">
         <v>962</v>
       </c>
-      <c r="H7" s="279" t="s">
+      <c r="H7" s="283" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="59" customFormat="1" ht="30" customHeight="1">
-      <c r="A8" s="279"/>
-      <c r="B8" s="279"/>
+      <c r="A8" s="283"/>
+      <c r="B8" s="283"/>
       <c r="C8" s="253" t="s">
         <v>6</v>
       </c>
@@ -26958,8 +26944,8 @@
       <c r="F8" s="253" t="s">
         <v>958</v>
       </c>
-      <c r="G8" s="279"/>
-      <c r="H8" s="279"/>
+      <c r="G8" s="283"/>
+      <c r="H8" s="283"/>
     </row>
     <row r="9" spans="1:9" s="64" customFormat="1" ht="30" customHeight="1">
       <c r="A9" s="77"/>
@@ -27028,7 +27014,7 @@
       <c r="I14" s="87"/>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I8" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A9:I9" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <mergeCells count="9">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -27072,43 +27058,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="60" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="282" t="s">
+      <c r="A1" s="286" t="s">
         <v>988</v>
       </c>
-      <c r="B1" s="282"/>
-      <c r="C1" s="282"/>
-      <c r="D1" s="282"/>
-      <c r="E1" s="282"/>
-      <c r="F1" s="282"/>
-      <c r="G1" s="282"/>
-      <c r="H1" s="282"/>
-      <c r="I1" s="283"/>
+      <c r="B1" s="286"/>
+      <c r="C1" s="286"/>
+      <c r="D1" s="286"/>
+      <c r="E1" s="286"/>
+      <c r="F1" s="286"/>
+      <c r="G1" s="286"/>
+      <c r="H1" s="286"/>
+      <c r="I1" s="286"/>
     </row>
     <row r="2" spans="1:11" s="60" customFormat="1" ht="30" customHeight="1">
-      <c r="A2" s="282" t="s">
+      <c r="A2" s="286" t="s">
         <v>983</v>
       </c>
-      <c r="B2" s="282"/>
-      <c r="C2" s="282"/>
-      <c r="D2" s="282"/>
-      <c r="E2" s="282"/>
-      <c r="F2" s="282"/>
-      <c r="G2" s="282"/>
-      <c r="H2" s="282"/>
-      <c r="I2" s="283"/>
+      <c r="B2" s="286"/>
+      <c r="C2" s="286"/>
+      <c r="D2" s="286"/>
+      <c r="E2" s="286"/>
+      <c r="F2" s="286"/>
+      <c r="G2" s="286"/>
+      <c r="H2" s="286"/>
+      <c r="I2" s="286"/>
     </row>
     <row r="3" spans="1:11" s="60" customFormat="1" ht="30" customHeight="1">
-      <c r="A3" s="282" t="s">
+      <c r="A3" s="286" t="s">
         <v>1017</v>
       </c>
-      <c r="B3" s="282"/>
-      <c r="C3" s="282"/>
-      <c r="D3" s="282"/>
-      <c r="E3" s="282"/>
-      <c r="F3" s="282"/>
-      <c r="G3" s="282"/>
-      <c r="H3" s="282"/>
-      <c r="I3" s="283"/>
+      <c r="B3" s="286"/>
+      <c r="C3" s="286"/>
+      <c r="D3" s="286"/>
+      <c r="E3" s="286"/>
+      <c r="F3" s="286"/>
+      <c r="G3" s="286"/>
+      <c r="H3" s="286"/>
+      <c r="I3" s="286"/>
     </row>
     <row r="4" spans="1:11" s="60" customFormat="1" ht="30" customHeight="1">
       <c r="A4" s="91" t="s">
@@ -27125,11 +27111,11 @@
       <c r="G4" s="97" t="s">
         <v>967</v>
       </c>
-      <c r="H4" s="285">
+      <c r="H4" s="287">
         <f>'Company information'!D8</f>
         <v>0</v>
       </c>
-      <c r="I4" s="286"/>
+      <c r="I4" s="287"/>
     </row>
     <row r="5" spans="1:11" s="60" customFormat="1" ht="30" customHeight="1">
       <c r="A5" s="91" t="s">
@@ -27144,11 +27130,11 @@
       <c r="E5" s="95"/>
       <c r="F5" s="94"/>
       <c r="G5" s="98"/>
-      <c r="H5" s="285">
+      <c r="H5" s="287">
         <f>'Company information'!E8</f>
         <v>0</v>
       </c>
-      <c r="I5" s="286"/>
+      <c r="I5" s="287"/>
     </row>
     <row r="6" spans="1:11" s="60" customFormat="1" ht="30" customHeight="1">
       <c r="A6" s="99">
@@ -27160,58 +27146,58 @@
       <c r="D6" s="94"/>
       <c r="E6" s="95"/>
       <c r="F6" s="96"/>
-      <c r="G6" s="75" t="s">
+      <c r="G6" s="280" t="s">
         <v>968</v>
       </c>
-      <c r="H6" s="287">
+      <c r="H6" s="401">
         <f>'Company information'!H9</f>
         <v>0</v>
       </c>
-      <c r="I6" s="288"/>
+      <c r="I6" s="401"/>
     </row>
     <row r="7" spans="1:11" s="59" customFormat="1" ht="30" customHeight="1">
-      <c r="A7" s="289" t="s">
+      <c r="A7" s="288" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="289" t="s">
+      <c r="B7" s="288" t="s">
         <v>760</v>
       </c>
-      <c r="C7" s="291" t="s">
+      <c r="C7" s="288" t="s">
         <v>992</v>
       </c>
-      <c r="D7" s="292"/>
-      <c r="E7" s="291" t="s">
+      <c r="D7" s="288"/>
+      <c r="E7" s="288" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="292"/>
-      <c r="G7" s="293" t="s">
+      <c r="F7" s="288"/>
+      <c r="G7" s="288" t="s">
         <v>962</v>
       </c>
-      <c r="H7" s="290" t="s">
+      <c r="H7" s="289" t="s">
         <v>1018</v>
       </c>
-      <c r="I7" s="284" t="s">
+      <c r="I7" s="288" t="s">
         <v>1048</v>
       </c>
     </row>
     <row r="8" spans="1:11" s="59" customFormat="1" ht="30" customHeight="1">
-      <c r="A8" s="289"/>
-      <c r="B8" s="289"/>
-      <c r="C8" s="254" t="s">
+      <c r="A8" s="288"/>
+      <c r="B8" s="288"/>
+      <c r="C8" s="281" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="254" t="s">
+      <c r="D8" s="281" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="254" t="s">
+      <c r="E8" s="281" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="254" t="s">
+      <c r="F8" s="281" t="s">
         <v>958</v>
       </c>
-      <c r="G8" s="294"/>
-      <c r="H8" s="289"/>
-      <c r="I8" s="284"/>
+      <c r="G8" s="288"/>
+      <c r="H8" s="288"/>
+      <c r="I8" s="288"/>
       <c r="J8" s="277"/>
       <c r="K8" s="277"/>
     </row>
@@ -27227,17 +27213,17 @@
       <c r="I9" s="100"/>
     </row>
     <row r="10" spans="1:11" s="64" customFormat="1" ht="30" customHeight="1">
-      <c r="A10" s="280" t="s">
+      <c r="A10" s="284" t="s">
         <v>1020</v>
       </c>
-      <c r="B10" s="281"/>
-      <c r="C10" s="281"/>
-      <c r="D10" s="281"/>
-      <c r="E10" s="281"/>
-      <c r="F10" s="281"/>
-      <c r="G10" s="281"/>
-      <c r="H10" s="281"/>
-      <c r="I10" s="281"/>
+      <c r="B10" s="285"/>
+      <c r="C10" s="285"/>
+      <c r="D10" s="285"/>
+      <c r="E10" s="285"/>
+      <c r="F10" s="285"/>
+      <c r="G10" s="285"/>
+      <c r="H10" s="285"/>
+      <c r="I10" s="285"/>
     </row>
   </sheetData>
   <autoFilter ref="A9:K9" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
@@ -27269,7 +27255,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB6F532-92EF-483A-99A9-EF9B2ABC7956}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:AS8"/>
+  <dimension ref="A1:AT9"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="12" style="258" customWidth="1"/>
@@ -27281,71 +27267,71 @@
     <col min="7" max="7" width="16.109375" style="258" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="7.77734375" style="258" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="23.5546875" style="258" customWidth="1"/>
-    <col min="10" max="10" width="22.33203125" style="258" customWidth="1"/>
-    <col min="11" max="12" width="21.77734375" style="258" customWidth="1"/>
-    <col min="13" max="13" width="15" style="258" customWidth="1"/>
-    <col min="14" max="14" width="11.77734375" style="258" customWidth="1"/>
-    <col min="15" max="15" width="12.5546875" style="258" customWidth="1"/>
-    <col min="16" max="16" width="19.109375" style="258" customWidth="1"/>
-    <col min="17" max="17" width="16.33203125" style="258" customWidth="1"/>
-    <col min="18" max="18" width="15.109375" style="258" customWidth="1"/>
-    <col min="19" max="19" width="18.109375" style="258" customWidth="1"/>
-    <col min="20" max="20" width="16.33203125" style="258" customWidth="1"/>
-    <col min="21" max="21" width="30.5546875" style="258" customWidth="1"/>
-    <col min="22" max="22" width="19.33203125" style="258" customWidth="1"/>
-    <col min="23" max="23" width="14" style="258" customWidth="1"/>
-    <col min="24" max="24" width="14.109375" style="258" customWidth="1"/>
-    <col min="25" max="25" width="26.109375" style="258" customWidth="1"/>
-    <col min="26" max="26" width="27.109375" style="258" customWidth="1"/>
-    <col min="27" max="27" width="15.33203125" style="258" customWidth="1"/>
-    <col min="28" max="28" width="23" style="258" customWidth="1"/>
-    <col min="29" max="29" width="22.109375" style="258" customWidth="1"/>
-    <col min="30" max="30" width="20.109375" style="258" customWidth="1"/>
-    <col min="31" max="31" width="14.21875" style="258" customWidth="1"/>
-    <col min="32" max="32" width="18.44140625" style="258" customWidth="1"/>
-    <col min="33" max="33" width="26.6640625" style="258" customWidth="1"/>
-    <col min="34" max="34" width="14.77734375" style="258" customWidth="1"/>
-    <col min="35" max="35" width="17.77734375" style="258" customWidth="1"/>
-    <col min="36" max="36" width="26.44140625" style="258" customWidth="1"/>
-    <col min="37" max="37" width="28.6640625" style="258" customWidth="1"/>
-    <col min="38" max="38" width="17.6640625" style="258" customWidth="1"/>
-    <col min="39" max="39" width="28" style="258" customWidth="1"/>
-    <col min="40" max="40" width="27.21875" style="258" customWidth="1"/>
-    <col min="41" max="41" width="18.33203125" style="258" customWidth="1"/>
-    <col min="42" max="42" width="31.33203125" style="258" customWidth="1"/>
-    <col min="43" max="43" width="13.109375" style="258" customWidth="1"/>
-    <col min="44" max="44" width="8.109375" style="258" customWidth="1"/>
-    <col min="45" max="45" width="18.21875" style="258" customWidth="1"/>
-    <col min="46" max="16384" width="8.88671875" style="258"/>
+    <col min="10" max="11" width="22.33203125" style="258" customWidth="1"/>
+    <col min="12" max="13" width="21.77734375" style="258" customWidth="1"/>
+    <col min="14" max="14" width="15" style="258" customWidth="1"/>
+    <col min="15" max="15" width="11.77734375" style="258" customWidth="1"/>
+    <col min="16" max="16" width="12.5546875" style="258" customWidth="1"/>
+    <col min="17" max="17" width="19.109375" style="258" customWidth="1"/>
+    <col min="18" max="18" width="16.33203125" style="258" customWidth="1"/>
+    <col min="19" max="19" width="15.109375" style="258" customWidth="1"/>
+    <col min="20" max="20" width="18.109375" style="258" customWidth="1"/>
+    <col min="21" max="21" width="16.33203125" style="258" customWidth="1"/>
+    <col min="22" max="22" width="30.5546875" style="258" customWidth="1"/>
+    <col min="23" max="23" width="19.33203125" style="258" customWidth="1"/>
+    <col min="24" max="24" width="14" style="258" customWidth="1"/>
+    <col min="25" max="25" width="14.109375" style="258" customWidth="1"/>
+    <col min="26" max="26" width="26.109375" style="258" customWidth="1"/>
+    <col min="27" max="27" width="27.109375" style="258" customWidth="1"/>
+    <col min="28" max="28" width="15.33203125" style="258" customWidth="1"/>
+    <col min="29" max="29" width="23" style="258" customWidth="1"/>
+    <col min="30" max="30" width="22.109375" style="258" customWidth="1"/>
+    <col min="31" max="31" width="20.109375" style="258" customWidth="1"/>
+    <col min="32" max="32" width="14.21875" style="258" customWidth="1"/>
+    <col min="33" max="33" width="18.44140625" style="258" customWidth="1"/>
+    <col min="34" max="34" width="26.6640625" style="258" customWidth="1"/>
+    <col min="35" max="35" width="14.77734375" style="258" customWidth="1"/>
+    <col min="36" max="36" width="17.77734375" style="258" customWidth="1"/>
+    <col min="37" max="37" width="26.44140625" style="258" customWidth="1"/>
+    <col min="38" max="38" width="28.6640625" style="258" customWidth="1"/>
+    <col min="39" max="39" width="17.6640625" style="258" customWidth="1"/>
+    <col min="40" max="40" width="28" style="258" customWidth="1"/>
+    <col min="41" max="41" width="27.21875" style="258" customWidth="1"/>
+    <col min="42" max="42" width="18.33203125" style="258" customWidth="1"/>
+    <col min="43" max="43" width="31.33203125" style="258" customWidth="1"/>
+    <col min="44" max="44" width="17.88671875" style="258" customWidth="1"/>
+    <col min="45" max="45" width="29.6640625" style="258" customWidth="1"/>
+    <col min="46" max="46" width="18.21875" style="258" customWidth="1"/>
+    <col min="47" max="16384" width="8.88671875" style="258"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" ht="24.6">
-      <c r="A1" s="295" t="s">
+    <row r="1" spans="1:46" ht="24.6">
+      <c r="A1" s="299" t="s">
         <v>980</v>
       </c>
-      <c r="B1" s="295"/>
-      <c r="C1" s="295"/>
-      <c r="D1" s="295"/>
-      <c r="E1" s="295"/>
-      <c r="F1" s="295"/>
-      <c r="G1" s="295"/>
-      <c r="H1" s="295"/>
-      <c r="I1" s="295"/>
-      <c r="J1" s="295"/>
-      <c r="K1" s="295"/>
-      <c r="L1" s="295"/>
-      <c r="M1" s="295"/>
-      <c r="N1" s="295"/>
-      <c r="O1" s="295"/>
-      <c r="P1" s="295"/>
-      <c r="Q1" s="295"/>
-      <c r="R1" s="296"/>
-      <c r="S1" s="255"/>
+      <c r="B1" s="299"/>
+      <c r="C1" s="299"/>
+      <c r="D1" s="299"/>
+      <c r="E1" s="299"/>
+      <c r="F1" s="299"/>
+      <c r="G1" s="299"/>
+      <c r="H1" s="299"/>
+      <c r="I1" s="299"/>
+      <c r="J1" s="299"/>
+      <c r="K1" s="278"/>
+      <c r="L1" s="278"/>
+      <c r="M1" s="278"/>
+      <c r="N1" s="278"/>
+      <c r="O1" s="278"/>
+      <c r="P1" s="278"/>
+      <c r="Q1" s="278"/>
+      <c r="R1" s="278"/>
+      <c r="S1" s="279"/>
       <c r="T1" s="255"/>
       <c r="U1" s="255"/>
       <c r="V1" s="255"/>
       <c r="W1" s="255"/>
-      <c r="X1" s="256"/>
+      <c r="X1" s="255"/>
       <c r="Y1" s="256"/>
       <c r="Z1" s="256"/>
       <c r="AA1" s="256"/>
@@ -27357,7 +27343,7 @@
       <c r="AG1" s="256"/>
       <c r="AH1" s="256"/>
       <c r="AI1" s="256"/>
-      <c r="AJ1" s="255"/>
+      <c r="AJ1" s="256"/>
       <c r="AK1" s="255"/>
       <c r="AL1" s="255"/>
       <c r="AM1" s="255"/>
@@ -27366,35 +27352,36 @@
       <c r="AP1" s="255"/>
       <c r="AQ1" s="255"/>
       <c r="AR1" s="255"/>
-      <c r="AS1" s="257"/>
-    </row>
-    <row r="2" spans="1:45" ht="24.6">
-      <c r="A2" s="295" t="s">
+      <c r="AS1" s="255"/>
+      <c r="AT1" s="257"/>
+    </row>
+    <row r="2" spans="1:46" ht="24.6">
+      <c r="A2" s="299" t="s">
         <v>983</v>
       </c>
-      <c r="B2" s="295"/>
-      <c r="C2" s="295"/>
-      <c r="D2" s="295"/>
-      <c r="E2" s="295"/>
-      <c r="F2" s="295"/>
-      <c r="G2" s="295"/>
-      <c r="H2" s="295"/>
-      <c r="I2" s="295"/>
-      <c r="J2" s="295"/>
-      <c r="K2" s="295"/>
-      <c r="L2" s="295"/>
-      <c r="M2" s="295"/>
-      <c r="N2" s="295"/>
-      <c r="O2" s="295"/>
-      <c r="P2" s="295"/>
-      <c r="Q2" s="295"/>
-      <c r="R2" s="296"/>
-      <c r="S2" s="255"/>
+      <c r="B2" s="299"/>
+      <c r="C2" s="299"/>
+      <c r="D2" s="299"/>
+      <c r="E2" s="299"/>
+      <c r="F2" s="299"/>
+      <c r="G2" s="299"/>
+      <c r="H2" s="299"/>
+      <c r="I2" s="299"/>
+      <c r="J2" s="299"/>
+      <c r="K2" s="278"/>
+      <c r="L2" s="278"/>
+      <c r="M2" s="278"/>
+      <c r="N2" s="278"/>
+      <c r="O2" s="278"/>
+      <c r="P2" s="278"/>
+      <c r="Q2" s="278"/>
+      <c r="R2" s="278"/>
+      <c r="S2" s="279"/>
       <c r="T2" s="255"/>
       <c r="U2" s="255"/>
       <c r="V2" s="255"/>
       <c r="W2" s="255"/>
-      <c r="X2" s="256"/>
+      <c r="X2" s="255"/>
       <c r="Y2" s="256"/>
       <c r="Z2" s="256"/>
       <c r="AA2" s="256"/>
@@ -27406,7 +27393,7 @@
       <c r="AG2" s="256"/>
       <c r="AH2" s="256"/>
       <c r="AI2" s="256"/>
-      <c r="AJ2" s="255"/>
+      <c r="AJ2" s="256"/>
       <c r="AK2" s="255"/>
       <c r="AL2" s="255"/>
       <c r="AM2" s="255"/>
@@ -27415,35 +27402,36 @@
       <c r="AP2" s="255"/>
       <c r="AQ2" s="255"/>
       <c r="AR2" s="255"/>
-      <c r="AS2" s="257"/>
-    </row>
-    <row r="3" spans="1:45" ht="24.6">
-      <c r="A3" s="295" t="s">
+      <c r="AS2" s="255"/>
+      <c r="AT2" s="257"/>
+    </row>
+    <row r="3" spans="1:46" ht="24.6">
+      <c r="A3" s="299" t="s">
         <v>957</v>
       </c>
-      <c r="B3" s="295"/>
-      <c r="C3" s="295"/>
-      <c r="D3" s="295"/>
-      <c r="E3" s="295"/>
-      <c r="F3" s="295"/>
-      <c r="G3" s="295"/>
-      <c r="H3" s="295"/>
-      <c r="I3" s="295"/>
-      <c r="J3" s="295"/>
-      <c r="K3" s="295"/>
-      <c r="L3" s="295"/>
-      <c r="M3" s="295"/>
-      <c r="N3" s="295"/>
-      <c r="O3" s="295"/>
-      <c r="P3" s="295"/>
-      <c r="Q3" s="295"/>
-      <c r="R3" s="296"/>
-      <c r="S3" s="255"/>
+      <c r="B3" s="299"/>
+      <c r="C3" s="299"/>
+      <c r="D3" s="299"/>
+      <c r="E3" s="299"/>
+      <c r="F3" s="299"/>
+      <c r="G3" s="299"/>
+      <c r="H3" s="299"/>
+      <c r="I3" s="299"/>
+      <c r="J3" s="299"/>
+      <c r="K3" s="278"/>
+      <c r="L3" s="278"/>
+      <c r="M3" s="278"/>
+      <c r="N3" s="278"/>
+      <c r="O3" s="278"/>
+      <c r="P3" s="278"/>
+      <c r="Q3" s="278"/>
+      <c r="R3" s="278"/>
+      <c r="S3" s="279"/>
       <c r="T3" s="255"/>
       <c r="U3" s="255"/>
       <c r="V3" s="255"/>
       <c r="W3" s="255"/>
-      <c r="X3" s="256"/>
+      <c r="X3" s="255"/>
       <c r="Y3" s="256"/>
       <c r="Z3" s="256"/>
       <c r="AA3" s="256"/>
@@ -27455,7 +27443,7 @@
       <c r="AG3" s="256"/>
       <c r="AH3" s="256"/>
       <c r="AI3" s="256"/>
-      <c r="AJ3" s="255"/>
+      <c r="AJ3" s="256"/>
       <c r="AK3" s="255"/>
       <c r="AL3" s="255"/>
       <c r="AM3" s="255"/>
@@ -27464,9 +27452,10 @@
       <c r="AP3" s="255"/>
       <c r="AQ3" s="255"/>
       <c r="AR3" s="255"/>
-      <c r="AS3" s="257"/>
-    </row>
-    <row r="4" spans="1:45" ht="24.6">
+      <c r="AS3" s="255"/>
+      <c r="AT3" s="257"/>
+    </row>
+    <row r="4" spans="1:46" ht="24.6">
       <c r="A4" s="259" t="s">
         <v>969</v>
       </c>
@@ -27483,24 +27472,23 @@
       <c r="I4" s="265" t="s">
         <v>967</v>
       </c>
-      <c r="J4" s="255"/>
-      <c r="K4" s="266">
+      <c r="J4" s="266">
         <f>'Company information'!D8</f>
         <v>0</v>
       </c>
-      <c r="L4" s="266"/>
-      <c r="M4" s="267"/>
-      <c r="N4" s="266"/>
+      <c r="K4" s="255"/>
+      <c r="M4" s="266"/>
+      <c r="N4" s="267"/>
       <c r="O4" s="266"/>
       <c r="P4" s="266"/>
       <c r="Q4" s="266"/>
-      <c r="R4" s="256"/>
-      <c r="S4" s="255"/>
+      <c r="R4" s="266"/>
+      <c r="S4" s="256"/>
       <c r="T4" s="255"/>
       <c r="U4" s="255"/>
       <c r="V4" s="255"/>
       <c r="W4" s="255"/>
-      <c r="X4" s="256"/>
+      <c r="X4" s="255"/>
       <c r="Y4" s="256"/>
       <c r="Z4" s="256"/>
       <c r="AA4" s="256"/>
@@ -27512,7 +27500,7 @@
       <c r="AG4" s="256"/>
       <c r="AH4" s="256"/>
       <c r="AI4" s="256"/>
-      <c r="AJ4" s="255"/>
+      <c r="AJ4" s="256"/>
       <c r="AK4" s="255"/>
       <c r="AL4" s="255"/>
       <c r="AM4" s="255"/>
@@ -27521,9 +27509,10 @@
       <c r="AP4" s="255"/>
       <c r="AQ4" s="255"/>
       <c r="AR4" s="255"/>
-      <c r="AS4" s="257"/>
-    </row>
-    <row r="5" spans="1:45" ht="24.6">
+      <c r="AS4" s="255"/>
+      <c r="AT4" s="257"/>
+    </row>
+    <row r="5" spans="1:46" ht="24.6">
       <c r="A5" s="268" t="s">
         <v>984</v>
       </c>
@@ -27538,53 +27527,53 @@
       <c r="G5" s="264"/>
       <c r="H5" s="264"/>
       <c r="I5" s="255"/>
-      <c r="J5" s="255"/>
-      <c r="K5" s="266">
+      <c r="J5" s="266">
         <f>'Company information'!E8</f>
         <v>0</v>
       </c>
-      <c r="L5" s="266"/>
-      <c r="M5" s="267"/>
-      <c r="N5" s="298" t="s">
+      <c r="K5" s="255"/>
+      <c r="M5" s="266"/>
+      <c r="N5" s="267"/>
+      <c r="O5" s="301" t="s">
         <v>1013</v>
       </c>
-      <c r="O5" s="298"/>
-      <c r="P5" s="298"/>
-      <c r="Q5" s="298"/>
-      <c r="R5" s="298"/>
-      <c r="S5" s="298"/>
-      <c r="T5" s="298"/>
-      <c r="U5" s="299"/>
-      <c r="V5" s="297" t="s">
+      <c r="P5" s="301"/>
+      <c r="Q5" s="301"/>
+      <c r="R5" s="301"/>
+      <c r="S5" s="301"/>
+      <c r="T5" s="301"/>
+      <c r="U5" s="301"/>
+      <c r="V5" s="302"/>
+      <c r="W5" s="300" t="s">
         <v>1016</v>
       </c>
-      <c r="W5" s="297"/>
-      <c r="X5" s="302" t="s">
+      <c r="X5" s="300"/>
+      <c r="Y5" s="308" t="s">
         <v>1015</v>
       </c>
-      <c r="Y5" s="302"/>
-      <c r="Z5" s="302"/>
-      <c r="AA5" s="302"/>
-      <c r="AB5" s="302"/>
-      <c r="AC5" s="302"/>
-      <c r="AD5" s="302"/>
-      <c r="AE5" s="302"/>
-      <c r="AF5" s="302"/>
-      <c r="AG5" s="302"/>
-      <c r="AH5" s="302"/>
-      <c r="AI5" s="302"/>
-      <c r="AJ5" s="302"/>
-      <c r="AK5" s="302"/>
-      <c r="AL5" s="302"/>
-      <c r="AM5" s="302"/>
-      <c r="AN5" s="302"/>
-      <c r="AO5" s="302"/>
-      <c r="AP5" s="302"/>
-      <c r="AQ5" s="302"/>
-      <c r="AR5" s="302"/>
-      <c r="AS5" s="302"/>
-    </row>
-    <row r="6" spans="1:45" ht="24.6">
+      <c r="Z5" s="308"/>
+      <c r="AA5" s="308"/>
+      <c r="AB5" s="308"/>
+      <c r="AC5" s="308"/>
+      <c r="AD5" s="308"/>
+      <c r="AE5" s="308"/>
+      <c r="AF5" s="308"/>
+      <c r="AG5" s="308"/>
+      <c r="AH5" s="308"/>
+      <c r="AI5" s="308"/>
+      <c r="AJ5" s="308"/>
+      <c r="AK5" s="308"/>
+      <c r="AL5" s="308"/>
+      <c r="AM5" s="308"/>
+      <c r="AN5" s="308"/>
+      <c r="AO5" s="308"/>
+      <c r="AP5" s="308"/>
+      <c r="AQ5" s="308"/>
+      <c r="AR5" s="308"/>
+      <c r="AS5" s="308"/>
+      <c r="AT5" s="308"/>
+    </row>
+    <row r="6" spans="1:46" ht="24.6">
       <c r="A6" s="269">
         <f>'Company information'!H8</f>
         <v>0</v>
@@ -27599,168 +27588,172 @@
       <c r="I6" s="270" t="s">
         <v>968</v>
       </c>
-      <c r="J6" s="303">
+      <c r="J6" s="272">
         <f>'Company information'!H9</f>
         <v>0</v>
       </c>
-      <c r="K6" s="303"/>
-      <c r="L6" s="271"/>
-      <c r="M6" s="272"/>
-      <c r="N6" s="300"/>
-      <c r="O6" s="300"/>
-      <c r="P6" s="300"/>
-      <c r="Q6" s="300"/>
-      <c r="R6" s="300"/>
-      <c r="S6" s="300"/>
-      <c r="T6" s="300"/>
-      <c r="U6" s="301"/>
-      <c r="V6" s="297"/>
-      <c r="W6" s="297"/>
-      <c r="X6" s="302"/>
-      <c r="Y6" s="302"/>
-      <c r="Z6" s="302"/>
-      <c r="AA6" s="302"/>
-      <c r="AB6" s="302"/>
-      <c r="AC6" s="302"/>
-      <c r="AD6" s="302"/>
-      <c r="AE6" s="302"/>
-      <c r="AF6" s="302"/>
-      <c r="AG6" s="302"/>
-      <c r="AH6" s="302"/>
-      <c r="AI6" s="302"/>
-      <c r="AJ6" s="302"/>
-      <c r="AK6" s="302"/>
-      <c r="AL6" s="302"/>
-      <c r="AM6" s="302"/>
-      <c r="AN6" s="302"/>
-      <c r="AO6" s="302"/>
-      <c r="AP6" s="302"/>
-      <c r="AQ6" s="302"/>
-      <c r="AR6" s="302"/>
-      <c r="AS6" s="302"/>
-    </row>
-    <row r="7" spans="1:45" ht="22.8">
-      <c r="A7" s="304" t="s">
+      <c r="K6" s="272"/>
+      <c r="L6" s="272"/>
+      <c r="M6" s="271"/>
+      <c r="N6" s="272"/>
+      <c r="O6" s="303"/>
+      <c r="P6" s="303"/>
+      <c r="Q6" s="303"/>
+      <c r="R6" s="303"/>
+      <c r="S6" s="303"/>
+      <c r="T6" s="303"/>
+      <c r="U6" s="303"/>
+      <c r="V6" s="304"/>
+      <c r="W6" s="300"/>
+      <c r="X6" s="300"/>
+      <c r="Y6" s="308"/>
+      <c r="Z6" s="308"/>
+      <c r="AA6" s="308"/>
+      <c r="AB6" s="308"/>
+      <c r="AC6" s="308"/>
+      <c r="AD6" s="308"/>
+      <c r="AE6" s="308"/>
+      <c r="AF6" s="308"/>
+      <c r="AG6" s="308"/>
+      <c r="AH6" s="308"/>
+      <c r="AI6" s="308"/>
+      <c r="AJ6" s="308"/>
+      <c r="AK6" s="308"/>
+      <c r="AL6" s="308"/>
+      <c r="AM6" s="308"/>
+      <c r="AN6" s="308"/>
+      <c r="AO6" s="308"/>
+      <c r="AP6" s="308"/>
+      <c r="AQ6" s="308"/>
+      <c r="AR6" s="308"/>
+      <c r="AS6" s="308"/>
+      <c r="AT6" s="308"/>
+    </row>
+    <row r="7" spans="1:46" ht="22.8">
+      <c r="A7" s="309" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="304" t="s">
+      <c r="B7" s="309" t="s">
         <v>760</v>
       </c>
-      <c r="C7" s="304" t="s">
+      <c r="C7" s="309" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="305" t="s">
+      <c r="D7" s="294" t="s">
         <v>759</v>
       </c>
-      <c r="E7" s="304" t="s">
+      <c r="E7" s="309" t="s">
         <v>734</v>
       </c>
-      <c r="F7" s="304"/>
-      <c r="G7" s="304" t="s">
+      <c r="F7" s="309"/>
+      <c r="G7" s="309" t="s">
         <v>981</v>
       </c>
-      <c r="H7" s="304"/>
-      <c r="I7" s="304"/>
-      <c r="J7" s="305" t="s">
+      <c r="H7" s="309"/>
+      <c r="I7" s="309"/>
+      <c r="J7" s="294" t="s">
         <v>995</v>
       </c>
-      <c r="K7" s="306" t="s">
+      <c r="K7" s="297" t="s">
+        <v>1054</v>
+      </c>
+      <c r="L7" s="297" t="s">
         <v>1049</v>
       </c>
-      <c r="L7" s="306" t="s">
+      <c r="M7" s="297" t="s">
         <v>1053</v>
       </c>
-      <c r="M7" s="305" t="s">
+      <c r="N7" s="294" t="s">
         <v>996</v>
       </c>
-      <c r="N7" s="311"/>
-      <c r="O7" s="312"/>
-      <c r="P7" s="313"/>
-      <c r="Q7" s="308" t="s">
+      <c r="O7" s="305"/>
+      <c r="P7" s="306"/>
+      <c r="Q7" s="307"/>
+      <c r="R7" s="295" t="s">
         <v>1035</v>
       </c>
-      <c r="R7" s="308" t="s">
+      <c r="S7" s="295" t="s">
         <v>1036</v>
       </c>
-      <c r="S7" s="305" t="s">
+      <c r="T7" s="294" t="s">
         <v>1002</v>
       </c>
-      <c r="T7" s="305" t="s">
+      <c r="U7" s="294" t="s">
         <v>1001</v>
       </c>
-      <c r="U7" s="305" t="s">
+      <c r="V7" s="294" t="s">
         <v>1012</v>
       </c>
-      <c r="V7" s="305" t="s">
+      <c r="W7" s="294" t="s">
         <v>1014</v>
       </c>
-      <c r="W7" s="308" t="s">
+      <c r="X7" s="295" t="s">
         <v>1000</v>
       </c>
-      <c r="X7" s="308" t="s">
+      <c r="Y7" s="295" t="s">
         <v>1022</v>
       </c>
-      <c r="Y7" s="308" t="s">
+      <c r="Z7" s="295" t="s">
         <v>1023</v>
       </c>
-      <c r="Z7" s="308" t="s">
+      <c r="AA7" s="295" t="s">
         <v>1003</v>
       </c>
-      <c r="AA7" s="308" t="s">
+      <c r="AB7" s="295" t="s">
         <v>758</v>
       </c>
-      <c r="AB7" s="309"/>
-      <c r="AC7" s="309"/>
-      <c r="AD7" s="308" t="s">
+      <c r="AC7" s="296"/>
+      <c r="AD7" s="296"/>
+      <c r="AE7" s="295" t="s">
         <v>1004</v>
       </c>
-      <c r="AE7" s="308" t="s">
+      <c r="AF7" s="295" t="s">
         <v>1005</v>
       </c>
-      <c r="AF7" s="309"/>
-      <c r="AG7" s="308" t="s">
+      <c r="AG7" s="296"/>
+      <c r="AH7" s="295" t="s">
         <v>1024</v>
       </c>
-      <c r="AH7" s="308" t="s">
+      <c r="AI7" s="295" t="s">
         <v>997</v>
       </c>
-      <c r="AI7" s="309"/>
-      <c r="AJ7" s="308" t="s">
+      <c r="AJ7" s="296"/>
+      <c r="AK7" s="295" t="s">
         <v>1025</v>
       </c>
-      <c r="AK7" s="308" t="s">
+      <c r="AL7" s="295" t="s">
         <v>1026</v>
       </c>
-      <c r="AL7" s="308" t="s">
+      <c r="AM7" s="295" t="s">
         <v>1027</v>
       </c>
-      <c r="AM7" s="308" t="s">
+      <c r="AN7" s="295" t="s">
         <v>1028</v>
       </c>
-      <c r="AN7" s="308" t="s">
+      <c r="AO7" s="295" t="s">
         <v>1029</v>
       </c>
-      <c r="AO7" s="308" t="s">
+      <c r="AP7" s="295" t="s">
         <v>1030</v>
       </c>
-      <c r="AP7" s="308" t="s">
+      <c r="AQ7" s="295" t="s">
         <v>1031</v>
       </c>
-      <c r="AQ7" s="308" t="s">
+      <c r="AR7" s="295" t="s">
         <v>1032</v>
       </c>
-      <c r="AR7" s="308" t="s">
+      <c r="AS7" s="295" t="s">
         <v>760</v>
       </c>
-      <c r="AS7" s="308" t="s">
+      <c r="AT7" s="295" t="s">
         <v>1033</v>
       </c>
     </row>
-    <row r="8" spans="1:45" ht="22.8">
-      <c r="A8" s="304"/>
-      <c r="B8" s="304"/>
-      <c r="C8" s="304"/>
-      <c r="D8" s="305"/>
+    <row r="8" spans="1:46" ht="22.8">
+      <c r="A8" s="309"/>
+      <c r="B8" s="309"/>
+      <c r="C8" s="309"/>
+      <c r="D8" s="294"/>
       <c r="E8" s="273" t="s">
         <v>6</v>
       </c>
@@ -27776,109 +27769,111 @@
       <c r="I8" s="274" t="s">
         <v>960</v>
       </c>
-      <c r="J8" s="305"/>
-      <c r="K8" s="307"/>
-      <c r="L8" s="307"/>
-      <c r="M8" s="305"/>
-      <c r="N8" s="275" t="s">
+      <c r="J8" s="294"/>
+      <c r="K8" s="298"/>
+      <c r="L8" s="298"/>
+      <c r="M8" s="298"/>
+      <c r="N8" s="294"/>
+      <c r="O8" s="275" t="s">
         <v>1050</v>
       </c>
-      <c r="O8" s="275" t="s">
+      <c r="P8" s="275" t="s">
         <v>1051</v>
       </c>
-      <c r="P8" s="275" t="s">
+      <c r="Q8" s="275" t="s">
         <v>1052</v>
       </c>
-      <c r="Q8" s="309"/>
-      <c r="R8" s="309"/>
-      <c r="S8" s="305"/>
-      <c r="T8" s="305"/>
-      <c r="U8" s="305"/>
-      <c r="V8" s="305"/>
-      <c r="W8" s="310"/>
-      <c r="X8" s="309"/>
-      <c r="Y8" s="309"/>
-      <c r="Z8" s="309"/>
-      <c r="AA8" s="276" t="s">
+      <c r="R8" s="296"/>
+      <c r="S8" s="296"/>
+      <c r="T8" s="294"/>
+      <c r="U8" s="294"/>
+      <c r="V8" s="294"/>
+      <c r="W8" s="294"/>
+      <c r="X8" s="310"/>
+      <c r="Y8" s="296"/>
+      <c r="Z8" s="296"/>
+      <c r="AA8" s="296"/>
+      <c r="AB8" s="276" t="s">
         <v>1006</v>
       </c>
-      <c r="AB8" s="276" t="s">
+      <c r="AC8" s="276" t="s">
         <v>1034</v>
       </c>
-      <c r="AC8" s="276" t="s">
+      <c r="AD8" s="276" t="s">
         <v>1007</v>
       </c>
-      <c r="AD8" s="309"/>
-      <c r="AE8" s="276" t="s">
+      <c r="AE8" s="296"/>
+      <c r="AF8" s="276" t="s">
         <v>1008</v>
       </c>
-      <c r="AF8" s="276" t="s">
+      <c r="AG8" s="276" t="s">
         <v>1009</v>
       </c>
-      <c r="AG8" s="309"/>
-      <c r="AH8" s="276" t="s">
+      <c r="AH8" s="296"/>
+      <c r="AI8" s="276" t="s">
         <v>1010</v>
       </c>
-      <c r="AI8" s="276" t="s">
+      <c r="AJ8" s="276" t="s">
         <v>1011</v>
       </c>
-      <c r="AJ8" s="309"/>
-      <c r="AK8" s="309"/>
-      <c r="AL8" s="309"/>
-      <c r="AM8" s="309"/>
-      <c r="AN8" s="309"/>
-      <c r="AO8" s="309"/>
-      <c r="AP8" s="309"/>
-      <c r="AQ8" s="309"/>
-      <c r="AR8" s="309"/>
-      <c r="AS8" s="309"/>
-    </row>
+      <c r="AK8" s="296"/>
+      <c r="AL8" s="296"/>
+      <c r="AM8" s="296"/>
+      <c r="AN8" s="296"/>
+      <c r="AO8" s="296"/>
+      <c r="AP8" s="296"/>
+      <c r="AQ8" s="296"/>
+      <c r="AR8" s="296"/>
+      <c r="AS8" s="296"/>
+      <c r="AT8" s="296"/>
+    </row>
+    <row r="9" spans="1:46" ht="24.6" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A8:AS8" xr:uid="{8AB6F532-92EF-483A-99A9-EF9B2ABC7956}"/>
+  <autoFilter ref="A9:AT9" xr:uid="{8AB6F532-92EF-483A-99A9-EF9B2ABC7956}"/>
   <mergeCells count="43">
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="AO7:AO8"/>
-    <mergeCell ref="AP7:AP8"/>
     <mergeCell ref="AQ7:AQ8"/>
-    <mergeCell ref="AM7:AM8"/>
     <mergeCell ref="AR7:AR8"/>
-    <mergeCell ref="AS7:AS8"/>
-    <mergeCell ref="U7:U8"/>
+    <mergeCell ref="AN7:AN8"/>
+    <mergeCell ref="AT7:AT8"/>
     <mergeCell ref="V7:V8"/>
     <mergeCell ref="W7:W8"/>
-    <mergeCell ref="AN7:AN8"/>
+    <mergeCell ref="X7:X8"/>
+    <mergeCell ref="AO7:AO8"/>
+    <mergeCell ref="Z7:Z8"/>
+    <mergeCell ref="AA7:AA8"/>
+    <mergeCell ref="AB7:AD7"/>
+    <mergeCell ref="AE7:AE8"/>
+    <mergeCell ref="AF7:AG7"/>
+    <mergeCell ref="AH7:AH8"/>
+    <mergeCell ref="AI7:AJ7"/>
+    <mergeCell ref="AK7:AK8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="R7:R8"/>
     <mergeCell ref="Y7:Y8"/>
-    <mergeCell ref="Z7:Z8"/>
-    <mergeCell ref="AA7:AC7"/>
-    <mergeCell ref="AD7:AD8"/>
-    <mergeCell ref="AE7:AF7"/>
-    <mergeCell ref="AG7:AG8"/>
-    <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="AJ7:AJ8"/>
-    <mergeCell ref="AK7:AK8"/>
-    <mergeCell ref="AL7:AL8"/>
-    <mergeCell ref="X5:AS6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="S7:S8"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="G7:I7"/>
-    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="U7:U8"/>
+    <mergeCell ref="AS7:AS8"/>
     <mergeCell ref="K7:K8"/>
-    <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="X7:X8"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="W5:X6"/>
+    <mergeCell ref="O5:V6"/>
+    <mergeCell ref="O7:Q7"/>
     <mergeCell ref="M7:M8"/>
-    <mergeCell ref="R7:R8"/>
-    <mergeCell ref="S7:S8"/>
-    <mergeCell ref="T7:T8"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="V5:W6"/>
-    <mergeCell ref="N5:U6"/>
+    <mergeCell ref="AL7:AL8"/>
+    <mergeCell ref="AM7:AM8"/>
+    <mergeCell ref="AP7:AP8"/>
+    <mergeCell ref="Y5:AT6"/>
+    <mergeCell ref="A7:A8"/>
   </mergeCells>
   <phoneticPr fontId="71" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -27904,31 +27899,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="70" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="278" t="s">
+      <c r="A1" s="282" t="s">
         <v>987</v>
       </c>
-      <c r="B1" s="278"/>
-      <c r="C1" s="278"/>
-      <c r="D1" s="278"/>
-      <c r="E1" s="278"/>
+      <c r="B1" s="282"/>
+      <c r="C1" s="282"/>
+      <c r="D1" s="282"/>
+      <c r="E1" s="282"/>
     </row>
     <row r="2" spans="1:5" s="70" customFormat="1" ht="30" customHeight="1">
-      <c r="A2" s="278" t="s">
+      <c r="A2" s="282" t="s">
         <v>998</v>
       </c>
-      <c r="B2" s="278"/>
-      <c r="C2" s="278"/>
-      <c r="D2" s="278"/>
-      <c r="E2" s="278"/>
+      <c r="B2" s="282"/>
+      <c r="C2" s="282"/>
+      <c r="D2" s="282"/>
+      <c r="E2" s="282"/>
     </row>
     <row r="3" spans="1:5" s="70" customFormat="1" ht="30" customHeight="1">
-      <c r="A3" s="278" t="s">
+      <c r="A3" s="282" t="s">
         <v>999</v>
       </c>
-      <c r="B3" s="278"/>
-      <c r="C3" s="278"/>
-      <c r="D3" s="278"/>
-      <c r="E3" s="278"/>
+      <c r="B3" s="282"/>
+      <c r="C3" s="282"/>
+      <c r="D3" s="282"/>
+      <c r="E3" s="282"/>
     </row>
     <row r="4" spans="1:5" s="70" customFormat="1" ht="30" customHeight="1">
       <c r="A4" s="73" t="s">
@@ -27977,30 +27972,30 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" customHeight="1">
-      <c r="A7" s="279" t="s">
+      <c r="A7" s="283" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="279" t="s">
+      <c r="B7" s="283" t="s">
         <v>760</v>
       </c>
-      <c r="C7" s="279" t="s">
+      <c r="C7" s="283" t="s">
         <v>994</v>
       </c>
-      <c r="D7" s="279"/>
-      <c r="E7" s="279" t="s">
+      <c r="D7" s="283"/>
+      <c r="E7" s="283" t="s">
         <v>965</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1">
-      <c r="A8" s="279"/>
-      <c r="B8" s="279"/>
+      <c r="A8" s="283"/>
+      <c r="B8" s="283"/>
       <c r="C8" s="253" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="253" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="279"/>
+      <c r="E8" s="283"/>
     </row>
     <row r="9" spans="1:5" s="64" customFormat="1" ht="30" customHeight="1">
       <c r="A9" s="77"/>
@@ -28096,7 +28091,7 @@
       <c r="E21" s="50"/>
     </row>
   </sheetData>
-  <autoFilter ref="A8:E8" xr:uid="{00000000-0001-0000-0600-000000000000}"/>
+  <autoFilter ref="A9:E9" xr:uid="{00000000-0001-0000-0600-000000000000}"/>
   <mergeCells count="7">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C7:D7"/>
@@ -28137,44 +28132,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="102" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="314" t="s">
+      <c r="A1" s="311" t="s">
         <v>986</v>
       </c>
-      <c r="B1" s="314"/>
-      <c r="C1" s="314"/>
-      <c r="D1" s="314"/>
-      <c r="E1" s="314"/>
-      <c r="F1" s="314"/>
-      <c r="G1" s="314"/>
-      <c r="H1" s="314"/>
+      <c r="B1" s="311"/>
+      <c r="C1" s="311"/>
+      <c r="D1" s="311"/>
+      <c r="E1" s="311"/>
+      <c r="F1" s="311"/>
+      <c r="G1" s="311"/>
+      <c r="H1" s="311"/>
       <c r="I1" s="105"/>
       <c r="J1" s="105"/>
     </row>
     <row r="2" spans="1:14" s="102" customFormat="1" ht="30" customHeight="1">
-      <c r="A2" s="314" t="s">
+      <c r="A2" s="311" t="s">
         <v>990</v>
       </c>
-      <c r="B2" s="314"/>
-      <c r="C2" s="314"/>
-      <c r="D2" s="314"/>
-      <c r="E2" s="314"/>
-      <c r="F2" s="314"/>
-      <c r="G2" s="314"/>
-      <c r="H2" s="314"/>
+      <c r="B2" s="311"/>
+      <c r="C2" s="311"/>
+      <c r="D2" s="311"/>
+      <c r="E2" s="311"/>
+      <c r="F2" s="311"/>
+      <c r="G2" s="311"/>
+      <c r="H2" s="311"/>
       <c r="I2" s="105"/>
       <c r="J2" s="105"/>
     </row>
     <row r="3" spans="1:14" s="102" customFormat="1" ht="30" customHeight="1">
-      <c r="A3" s="314" t="s">
+      <c r="A3" s="311" t="s">
         <v>985</v>
       </c>
-      <c r="B3" s="314"/>
-      <c r="C3" s="314"/>
-      <c r="D3" s="314"/>
-      <c r="E3" s="314"/>
-      <c r="F3" s="314"/>
-      <c r="G3" s="314"/>
-      <c r="H3" s="314"/>
+      <c r="B3" s="311"/>
+      <c r="C3" s="311"/>
+      <c r="D3" s="311"/>
+      <c r="E3" s="311"/>
+      <c r="F3" s="311"/>
+      <c r="G3" s="311"/>
+      <c r="H3" s="311"/>
       <c r="I3" s="105"/>
       <c r="J3" s="105"/>
     </row>
@@ -28233,42 +28228,42 @@
       <c r="J6" s="101"/>
     </row>
     <row r="7" spans="1:14" s="59" customFormat="1" ht="30" customHeight="1">
-      <c r="A7" s="289" t="s">
+      <c r="A7" s="288" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="289" t="s">
+      <c r="B7" s="288" t="s">
         <v>760</v>
       </c>
-      <c r="C7" s="291" t="s">
+      <c r="C7" s="290" t="s">
         <v>734</v>
       </c>
-      <c r="D7" s="292"/>
-      <c r="E7" s="293" t="s">
+      <c r="D7" s="291"/>
+      <c r="E7" s="292" t="s">
         <v>963</v>
       </c>
-      <c r="F7" s="293" t="s">
+      <c r="F7" s="292" t="s">
         <v>961</v>
       </c>
-      <c r="G7" s="293" t="s">
+      <c r="G7" s="292" t="s">
         <v>964</v>
       </c>
-      <c r="H7" s="289" t="s">
+      <c r="H7" s="288" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:14" s="59" customFormat="1" ht="30" customHeight="1">
-      <c r="A8" s="289"/>
-      <c r="B8" s="289"/>
+      <c r="A8" s="288"/>
+      <c r="B8" s="288"/>
       <c r="C8" s="254" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="254" t="s">
         <v>958</v>
       </c>
-      <c r="E8" s="294"/>
-      <c r="F8" s="294"/>
-      <c r="G8" s="294"/>
-      <c r="H8" s="289"/>
+      <c r="E8" s="293"/>
+      <c r="F8" s="293"/>
+      <c r="G8" s="293"/>
+      <c r="H8" s="288"/>
     </row>
     <row r="9" spans="1:14" ht="30" customHeight="1">
       <c r="L9" s="111"/>
@@ -28296,7 +28291,7 @@
       <c r="N13" s="111"/>
     </row>
   </sheetData>
-  <autoFilter ref="A8:N8" xr:uid="{00000000-0001-0000-0700-000000000000}"/>
+  <autoFilter ref="A9:N9" xr:uid="{00000000-0001-0000-0700-000000000000}"/>
   <mergeCells count="10">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -28691,42 +28686,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.75" customHeight="1">
-      <c r="A1" s="337" t="s">
+      <c r="A1" s="334" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="337"/>
-      <c r="C1" s="337"/>
-      <c r="D1" s="337"/>
-      <c r="E1" s="337"/>
-      <c r="F1" s="337"/>
-      <c r="G1" s="337"/>
-      <c r="H1" s="337"/>
-      <c r="I1" s="337"/>
-      <c r="J1" s="337"/>
+      <c r="B1" s="334"/>
+      <c r="C1" s="334"/>
+      <c r="D1" s="334"/>
+      <c r="E1" s="334"/>
+      <c r="F1" s="334"/>
+      <c r="G1" s="334"/>
+      <c r="H1" s="334"/>
+      <c r="I1" s="334"/>
+      <c r="J1" s="334"/>
     </row>
     <row r="2" spans="1:10" ht="32.25" customHeight="1">
-      <c r="A2" s="337" t="s">
+      <c r="A2" s="334" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="337"/>
-      <c r="C2" s="337"/>
-      <c r="D2" s="337"/>
-      <c r="E2" s="337"/>
-      <c r="F2" s="337"/>
-      <c r="G2" s="337"/>
-      <c r="H2" s="337"/>
-      <c r="I2" s="337"/>
-      <c r="J2" s="337"/>
+      <c r="B2" s="334"/>
+      <c r="C2" s="334"/>
+      <c r="D2" s="334"/>
+      <c r="E2" s="334"/>
+      <c r="F2" s="334"/>
+      <c r="G2" s="334"/>
+      <c r="H2" s="334"/>
+      <c r="I2" s="334"/>
+      <c r="J2" s="334"/>
     </row>
     <row r="3" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A3" s="338" t="e">
+      <c r="A3" s="335" t="e">
         <f>'Annex I-IM State Charge'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B3" s="338"/>
-      <c r="C3" s="338"/>
-      <c r="D3" s="338"/>
-      <c r="E3" s="338"/>
+      <c r="B3" s="335"/>
+      <c r="C3" s="335"/>
+      <c r="D3" s="335"/>
+      <c r="E3" s="335"/>
       <c r="F3" s="120"/>
       <c r="G3" s="120"/>
       <c r="H3" s="120"/>
@@ -28734,13 +28729,13 @@
       <c r="J3" s="120"/>
     </row>
     <row r="4" spans="1:10" ht="21" customHeight="1">
-      <c r="A4" s="339" t="e">
+      <c r="A4" s="336" t="e">
         <f>'Annex I-IM State Charge'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B4" s="339"/>
-      <c r="C4" s="339"/>
-      <c r="D4" s="339"/>
+      <c r="B4" s="336"/>
+      <c r="C4" s="336"/>
+      <c r="D4" s="336"/>
       <c r="E4" s="120"/>
       <c r="F4" s="120"/>
       <c r="G4" s="120"/>
@@ -28749,47 +28744,47 @@
       <c r="J4" s="120"/>
     </row>
     <row r="5" spans="1:10" ht="24" customHeight="1">
-      <c r="A5" s="340" t="s">
+      <c r="A5" s="337" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="343" t="s">
+      <c r="B5" s="340" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="344"/>
-      <c r="D5" s="345"/>
-      <c r="E5" s="346" t="s">
+      <c r="C5" s="341"/>
+      <c r="D5" s="342"/>
+      <c r="E5" s="343" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="347"/>
-      <c r="G5" s="347"/>
-      <c r="H5" s="347"/>
-      <c r="I5" s="347"/>
-      <c r="J5" s="348" t="s">
+      <c r="F5" s="344"/>
+      <c r="G5" s="344"/>
+      <c r="H5" s="344"/>
+      <c r="I5" s="344"/>
+      <c r="J5" s="345" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="24" customHeight="1">
-      <c r="A6" s="341"/>
-      <c r="B6" s="351" t="s">
+      <c r="A6" s="338"/>
+      <c r="B6" s="348" t="s">
         <v>734</v>
       </c>
-      <c r="C6" s="352"/>
-      <c r="D6" s="353"/>
-      <c r="E6" s="354" t="s">
+      <c r="C6" s="349"/>
+      <c r="D6" s="350"/>
+      <c r="E6" s="351" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="355" t="s">
+      <c r="F6" s="352" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="351" t="s">
+      <c r="G6" s="348" t="s">
         <v>734</v>
       </c>
-      <c r="H6" s="352"/>
-      <c r="I6" s="353"/>
-      <c r="J6" s="349"/>
+      <c r="H6" s="349"/>
+      <c r="I6" s="350"/>
+      <c r="J6" s="346"/>
     </row>
     <row r="7" spans="1:10" ht="21" customHeight="1">
-      <c r="A7" s="342"/>
+      <c r="A7" s="339"/>
       <c r="B7" s="121" t="s">
         <v>6</v>
       </c>
@@ -28799,8 +28794,8 @@
       <c r="D7" s="121" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="355"/>
-      <c r="F7" s="355"/>
+      <c r="E7" s="352"/>
+      <c r="F7" s="352"/>
       <c r="G7" s="121" t="s">
         <v>6</v>
       </c>
@@ -28810,7 +28805,7 @@
       <c r="I7" s="121" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="350"/>
+      <c r="J7" s="347"/>
     </row>
     <row r="8" spans="1:10" ht="24" customHeight="1">
       <c r="A8" s="122">
@@ -29133,11 +29128,11 @@
       </c>
     </row>
     <row r="18" spans="1:10" ht="18" customHeight="1">
-      <c r="A18" s="336" t="s">
+      <c r="A18" s="333" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="336"/>
-      <c r="C18" s="336"/>
+      <c r="B18" s="333"/>
+      <c r="C18" s="333"/>
       <c r="D18" s="125">
         <f>SUM(D8:D17)</f>
         <v>717.92999999999984</v>
@@ -29155,11 +29150,11 @@
       <c r="J18" s="129"/>
     </row>
     <row r="19" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A19" s="336" t="s">
+      <c r="A19" s="333" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="336"/>
-      <c r="C19" s="336"/>
+      <c r="B19" s="333"/>
+      <c r="C19" s="333"/>
       <c r="D19" s="125"/>
       <c r="E19" s="126"/>
       <c r="F19" s="123"/>
@@ -29336,11 +29331,11 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="18" customHeight="1">
-      <c r="A25" s="336" t="s">
+      <c r="A25" s="333" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="336"/>
-      <c r="C25" s="336"/>
+      <c r="B25" s="333"/>
+      <c r="C25" s="333"/>
       <c r="D25" s="125">
         <f>SUM(D20:D24)</f>
         <v>363.15</v>
@@ -29358,11 +29353,11 @@
       <c r="J25" s="129"/>
     </row>
     <row r="26" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A26" s="336" t="s">
+      <c r="A26" s="333" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="336"/>
-      <c r="C26" s="336"/>
+      <c r="B26" s="333"/>
+      <c r="C26" s="333"/>
       <c r="D26" s="125"/>
       <c r="E26" s="126"/>
       <c r="F26" s="123"/>
@@ -29539,11 +29534,11 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="18" customHeight="1">
-      <c r="A32" s="336" t="s">
+      <c r="A32" s="333" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="336"/>
-      <c r="C32" s="336"/>
+      <c r="B32" s="333"/>
+      <c r="C32" s="333"/>
       <c r="D32" s="125">
         <f>SUM(D27:D31)</f>
         <v>424.63</v>
@@ -29561,11 +29556,11 @@
       <c r="J32" s="129"/>
     </row>
     <row r="33" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A33" s="336" t="s">
+      <c r="A33" s="333" t="s">
         <v>31</v>
       </c>
-      <c r="B33" s="336"/>
-      <c r="C33" s="336"/>
+      <c r="B33" s="333"/>
+      <c r="C33" s="333"/>
       <c r="D33" s="125"/>
       <c r="E33" s="126"/>
       <c r="F33" s="123"/>
@@ -29678,11 +29673,11 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="18" customHeight="1">
-      <c r="A37" s="336" t="s">
+      <c r="A37" s="333" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="336"/>
-      <c r="C37" s="336"/>
+      <c r="B37" s="333"/>
+      <c r="C37" s="333"/>
       <c r="D37" s="125">
         <f>SUM(D34:D36)</f>
         <v>323.32000000000005</v>
@@ -29700,11 +29695,11 @@
       <c r="J37" s="129"/>
     </row>
     <row r="38" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A38" s="336" t="s">
+      <c r="A38" s="333" t="s">
         <v>30</v>
       </c>
-      <c r="B38" s="336"/>
-      <c r="C38" s="336"/>
+      <c r="B38" s="333"/>
+      <c r="C38" s="333"/>
       <c r="D38" s="125"/>
       <c r="E38" s="126"/>
       <c r="F38" s="123"/>
@@ -29849,11 +29844,11 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="18" customHeight="1">
-      <c r="A43" s="336" t="s">
+      <c r="A43" s="333" t="s">
         <v>29</v>
       </c>
-      <c r="B43" s="336"/>
-      <c r="C43" s="336"/>
+      <c r="B43" s="333"/>
+      <c r="C43" s="333"/>
       <c r="D43" s="125">
         <f>SUM(D39:D42)</f>
         <v>272.76</v>
@@ -29871,11 +29866,11 @@
       <c r="J43" s="129"/>
     </row>
     <row r="44" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A44" s="336" t="s">
+      <c r="A44" s="333" t="s">
         <v>29</v>
       </c>
-      <c r="B44" s="336"/>
-      <c r="C44" s="336"/>
+      <c r="B44" s="333"/>
+      <c r="C44" s="333"/>
       <c r="D44" s="125"/>
       <c r="E44" s="126"/>
       <c r="F44" s="123"/>
@@ -30116,11 +30111,11 @@
       </c>
     </row>
     <row r="52" spans="1:10" ht="18" customHeight="1">
-      <c r="A52" s="336" t="s">
+      <c r="A52" s="333" t="s">
         <v>28</v>
       </c>
-      <c r="B52" s="336"/>
-      <c r="C52" s="336"/>
+      <c r="B52" s="333"/>
+      <c r="C52" s="333"/>
       <c r="D52" s="125">
         <f>SUM(D45:D51)</f>
         <v>462.51</v>
@@ -30138,11 +30133,11 @@
       <c r="J52" s="129"/>
     </row>
     <row r="53" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A53" s="336" t="s">
+      <c r="A53" s="333" t="s">
         <v>28</v>
       </c>
-      <c r="B53" s="336"/>
-      <c r="C53" s="336"/>
+      <c r="B53" s="333"/>
+      <c r="C53" s="333"/>
       <c r="D53" s="125"/>
       <c r="E53" s="126"/>
       <c r="F53" s="123"/>
@@ -30479,11 +30474,11 @@
       </c>
     </row>
     <row r="64" spans="1:10" ht="18" customHeight="1">
-      <c r="A64" s="336" t="s">
+      <c r="A64" s="333" t="s">
         <v>33</v>
       </c>
-      <c r="B64" s="336"/>
-      <c r="C64" s="336"/>
+      <c r="B64" s="333"/>
+      <c r="C64" s="333"/>
       <c r="D64" s="1">
         <f>SUM(D54:D63)</f>
         <v>1160.08</v>
@@ -30501,11 +30496,11 @@
       <c r="J64" s="129"/>
     </row>
     <row r="65" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A65" s="336" t="s">
+      <c r="A65" s="333" t="s">
         <v>33</v>
       </c>
-      <c r="B65" s="336"/>
-      <c r="C65" s="336"/>
+      <c r="B65" s="333"/>
+      <c r="C65" s="333"/>
       <c r="D65" s="1"/>
       <c r="E65" s="126"/>
       <c r="F65" s="123"/>
@@ -30778,11 +30773,11 @@
       </c>
     </row>
     <row r="74" spans="1:10" ht="18" customHeight="1">
-      <c r="A74" s="336" t="s">
+      <c r="A74" s="333" t="s">
         <v>34</v>
       </c>
-      <c r="B74" s="336"/>
-      <c r="C74" s="336"/>
+      <c r="B74" s="333"/>
+      <c r="C74" s="333"/>
       <c r="D74" s="1">
         <f>SUM(D66:D73)</f>
         <v>961.41000000000008</v>
@@ -30800,11 +30795,11 @@
       <c r="J74" s="129"/>
     </row>
     <row r="75" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A75" s="336" t="s">
+      <c r="A75" s="333" t="s">
         <v>34</v>
       </c>
-      <c r="B75" s="336"/>
-      <c r="C75" s="336"/>
+      <c r="B75" s="333"/>
+      <c r="C75" s="333"/>
       <c r="D75" s="1"/>
       <c r="E75" s="126"/>
       <c r="F75" s="123"/>
@@ -31109,11 +31104,11 @@
       </c>
     </row>
     <row r="85" spans="1:10" ht="18" customHeight="1">
-      <c r="A85" s="336" t="s">
+      <c r="A85" s="333" t="s">
         <v>35</v>
       </c>
-      <c r="B85" s="336"/>
-      <c r="C85" s="336"/>
+      <c r="B85" s="333"/>
+      <c r="C85" s="333"/>
       <c r="D85" s="1">
         <f>SUM(D76:D84)</f>
         <v>867.33999999999992</v>
@@ -31131,11 +31126,11 @@
       <c r="J85" s="129"/>
     </row>
     <row r="86" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A86" s="336" t="s">
+      <c r="A86" s="333" t="s">
         <v>35</v>
       </c>
-      <c r="B86" s="336"/>
-      <c r="C86" s="336"/>
+      <c r="B86" s="333"/>
+      <c r="C86" s="333"/>
       <c r="D86" s="1"/>
       <c r="E86" s="126"/>
       <c r="F86" s="123"/>
@@ -31472,11 +31467,11 @@
       </c>
     </row>
     <row r="97" spans="1:10" ht="18" customHeight="1">
-      <c r="A97" s="336" t="s">
+      <c r="A97" s="333" t="s">
         <v>20</v>
       </c>
-      <c r="B97" s="336"/>
-      <c r="C97" s="336"/>
+      <c r="B97" s="333"/>
+      <c r="C97" s="333"/>
       <c r="D97" s="1">
         <f>SUM(D87:D96)</f>
         <v>1138.25</v>
@@ -31494,11 +31489,11 @@
       <c r="J97" s="129"/>
     </row>
     <row r="98" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A98" s="336" t="s">
+      <c r="A98" s="333" t="s">
         <v>20</v>
       </c>
-      <c r="B98" s="336"/>
-      <c r="C98" s="336"/>
+      <c r="B98" s="333"/>
+      <c r="C98" s="333"/>
       <c r="D98" s="1"/>
       <c r="E98" s="126"/>
       <c r="F98" s="123"/>
@@ -31771,11 +31766,11 @@
       </c>
     </row>
     <row r="107" spans="1:10" ht="18" customHeight="1">
-      <c r="A107" s="336" t="s">
+      <c r="A107" s="333" t="s">
         <v>19</v>
       </c>
-      <c r="B107" s="336"/>
-      <c r="C107" s="336"/>
+      <c r="B107" s="333"/>
+      <c r="C107" s="333"/>
       <c r="D107" s="1">
         <f>SUM(D99:D106)</f>
         <v>585.41999999999996</v>
@@ -31793,11 +31788,11 @@
       <c r="J107" s="129"/>
     </row>
     <row r="108" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A108" s="336" t="s">
+      <c r="A108" s="333" t="s">
         <v>19</v>
       </c>
-      <c r="B108" s="336"/>
-      <c r="C108" s="336"/>
+      <c r="B108" s="333"/>
+      <c r="C108" s="333"/>
       <c r="D108" s="1"/>
       <c r="E108" s="126"/>
       <c r="F108" s="123"/>
@@ -32038,11 +32033,11 @@
       </c>
     </row>
     <row r="116" spans="1:10" ht="18" customHeight="1">
-      <c r="A116" s="336" t="s">
+      <c r="A116" s="333" t="s">
         <v>18</v>
       </c>
-      <c r="B116" s="336"/>
-      <c r="C116" s="336"/>
+      <c r="B116" s="333"/>
+      <c r="C116" s="333"/>
       <c r="D116" s="1">
         <f>SUM(D109:D115)</f>
         <v>744.72</v>
@@ -32060,11 +32055,11 @@
       <c r="J116" s="129"/>
     </row>
     <row r="117" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A117" s="336" t="s">
+      <c r="A117" s="333" t="s">
         <v>18</v>
       </c>
-      <c r="B117" s="336"/>
-      <c r="C117" s="336"/>
+      <c r="B117" s="333"/>
+      <c r="C117" s="333"/>
       <c r="D117" s="1"/>
       <c r="E117" s="126"/>
       <c r="F117" s="123"/>
@@ -32401,11 +32396,11 @@
       </c>
     </row>
     <row r="128" spans="1:10" ht="18" customHeight="1">
-      <c r="A128" s="336" t="s">
+      <c r="A128" s="333" t="s">
         <v>17</v>
       </c>
-      <c r="B128" s="336"/>
-      <c r="C128" s="336"/>
+      <c r="B128" s="333"/>
+      <c r="C128" s="333"/>
       <c r="D128" s="1">
         <f>SUM(D118:D127)</f>
         <v>1724.6699999999998</v>
@@ -32423,11 +32418,11 @@
       <c r="J128" s="129"/>
     </row>
     <row r="129" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A129" s="336" t="s">
+      <c r="A129" s="333" t="s">
         <v>17</v>
       </c>
-      <c r="B129" s="336"/>
-      <c r="C129" s="336"/>
+      <c r="B129" s="333"/>
+      <c r="C129" s="333"/>
       <c r="D129" s="1"/>
       <c r="E129" s="126"/>
       <c r="F129" s="123"/>
@@ -32604,11 +32599,11 @@
       </c>
     </row>
     <row r="135" spans="1:10" ht="18" customHeight="1">
-      <c r="A135" s="336" t="s">
+      <c r="A135" s="333" t="s">
         <v>21</v>
       </c>
-      <c r="B135" s="336"/>
-      <c r="C135" s="336"/>
+      <c r="B135" s="333"/>
+      <c r="C135" s="333"/>
       <c r="D135" s="1">
         <f>SUM(D130:D134)</f>
         <v>611.80000000000007</v>
@@ -32626,11 +32621,11 @@
       <c r="J135" s="129"/>
     </row>
     <row r="136" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A136" s="336" t="s">
+      <c r="A136" s="333" t="s">
         <v>21</v>
       </c>
-      <c r="B136" s="336"/>
-      <c r="C136" s="336"/>
+      <c r="B136" s="333"/>
+      <c r="C136" s="333"/>
       <c r="D136" s="1"/>
       <c r="E136" s="126"/>
       <c r="F136" s="123"/>
@@ -32967,11 +32962,11 @@
       </c>
     </row>
     <row r="147" spans="1:10" ht="18" customHeight="1">
-      <c r="A147" s="336" t="s">
+      <c r="A147" s="333" t="s">
         <v>22</v>
       </c>
-      <c r="B147" s="336"/>
-      <c r="C147" s="336"/>
+      <c r="B147" s="333"/>
+      <c r="C147" s="333"/>
       <c r="D147" s="1">
         <f>SUM(D137:D146)</f>
         <v>1337.1399999999999</v>
@@ -32989,11 +32984,11 @@
       <c r="J147" s="129"/>
     </row>
     <row r="148" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A148" s="336" t="s">
+      <c r="A148" s="333" t="s">
         <v>22</v>
       </c>
-      <c r="B148" s="336"/>
-      <c r="C148" s="336"/>
+      <c r="B148" s="333"/>
+      <c r="C148" s="333"/>
       <c r="D148" s="1"/>
       <c r="E148" s="126"/>
       <c r="F148" s="123"/>
@@ -33234,11 +33229,11 @@
       </c>
     </row>
     <row r="156" spans="1:10" ht="18" customHeight="1">
-      <c r="A156" s="336" t="s">
+      <c r="A156" s="333" t="s">
         <v>23</v>
       </c>
-      <c r="B156" s="336"/>
-      <c r="C156" s="336"/>
+      <c r="B156" s="333"/>
+      <c r="C156" s="333"/>
       <c r="D156" s="1">
         <f>SUM(D149:D155)</f>
         <v>868.96</v>
@@ -33256,11 +33251,11 @@
       <c r="J156" s="129"/>
     </row>
     <row r="157" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A157" s="336" t="s">
+      <c r="A157" s="333" t="s">
         <v>23</v>
       </c>
-      <c r="B157" s="336"/>
-      <c r="C157" s="336"/>
+      <c r="B157" s="333"/>
+      <c r="C157" s="333"/>
       <c r="D157" s="1"/>
       <c r="E157" s="126"/>
       <c r="F157" s="123"/>
@@ -33373,11 +33368,11 @@
       </c>
     </row>
     <row r="161" spans="1:10" ht="18" customHeight="1">
-      <c r="A161" s="336" t="s">
+      <c r="A161" s="333" t="s">
         <v>24</v>
       </c>
-      <c r="B161" s="336"/>
-      <c r="C161" s="336"/>
+      <c r="B161" s="333"/>
+      <c r="C161" s="333"/>
       <c r="D161" s="1">
         <f>SUM(D158:D160)</f>
         <v>308.44</v>
@@ -33395,11 +33390,11 @@
       <c r="J161" s="129"/>
     </row>
     <row r="162" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A162" s="336" t="s">
+      <c r="A162" s="333" t="s">
         <v>24</v>
       </c>
-      <c r="B162" s="336"/>
-      <c r="C162" s="336"/>
+      <c r="B162" s="333"/>
+      <c r="C162" s="333"/>
       <c r="D162" s="1"/>
       <c r="E162" s="126"/>
       <c r="F162" s="133"/>
@@ -33608,11 +33603,11 @@
       </c>
     </row>
     <row r="169" spans="1:10" ht="18" customHeight="1">
-      <c r="A169" s="336" t="s">
+      <c r="A169" s="333" t="s">
         <v>25</v>
       </c>
-      <c r="B169" s="336"/>
-      <c r="C169" s="336"/>
+      <c r="B169" s="333"/>
+      <c r="C169" s="333"/>
       <c r="D169" s="1">
         <f>SUM(D163:D168)</f>
         <v>845.91000000000008</v>
@@ -33630,11 +33625,11 @@
       <c r="J169" s="129"/>
     </row>
     <row r="170" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A170" s="336" t="s">
+      <c r="A170" s="333" t="s">
         <v>25</v>
       </c>
-      <c r="B170" s="336"/>
-      <c r="C170" s="336"/>
+      <c r="B170" s="333"/>
+      <c r="C170" s="333"/>
       <c r="D170" s="1"/>
       <c r="E170" s="126"/>
       <c r="F170" s="123"/>
@@ -33875,11 +33870,11 @@
       </c>
     </row>
     <row r="178" spans="1:10" ht="18" customHeight="1">
-      <c r="A178" s="336" t="s">
+      <c r="A178" s="333" t="s">
         <v>26</v>
       </c>
-      <c r="B178" s="336"/>
-      <c r="C178" s="336"/>
+      <c r="B178" s="333"/>
+      <c r="C178" s="333"/>
       <c r="D178" s="125">
         <f>SUM(D171:D177)</f>
         <v>757.07</v>
@@ -33897,11 +33892,11 @@
       <c r="J178" s="129"/>
     </row>
     <row r="179" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A179" s="336" t="s">
+      <c r="A179" s="333" t="s">
         <v>26</v>
       </c>
-      <c r="B179" s="336"/>
-      <c r="C179" s="336"/>
+      <c r="B179" s="333"/>
+      <c r="C179" s="333"/>
       <c r="D179" s="125"/>
       <c r="E179" s="126"/>
       <c r="F179" s="123"/>
@@ -34174,11 +34169,11 @@
       </c>
     </row>
     <row r="188" spans="1:10" ht="18" customHeight="1">
-      <c r="A188" s="336" t="s">
+      <c r="A188" s="333" t="s">
         <v>36</v>
       </c>
-      <c r="B188" s="336"/>
-      <c r="C188" s="336"/>
+      <c r="B188" s="333"/>
+      <c r="C188" s="333"/>
       <c r="D188" s="125">
         <f>SUM(D180:D187)</f>
         <v>1400.05</v>
@@ -34196,11 +34191,11 @@
       <c r="J188" s="129"/>
     </row>
     <row r="189" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A189" s="336" t="s">
+      <c r="A189" s="333" t="s">
         <v>36</v>
       </c>
-      <c r="B189" s="336"/>
-      <c r="C189" s="336"/>
+      <c r="B189" s="333"/>
+      <c r="C189" s="333"/>
       <c r="D189" s="125"/>
       <c r="E189" s="126"/>
       <c r="F189" s="123"/>
@@ -34441,11 +34436,11 @@
       </c>
     </row>
     <row r="197" spans="1:10" ht="18" customHeight="1">
-      <c r="A197" s="336" t="s">
+      <c r="A197" s="333" t="s">
         <v>37</v>
       </c>
-      <c r="B197" s="336"/>
-      <c r="C197" s="336"/>
+      <c r="B197" s="333"/>
+      <c r="C197" s="333"/>
       <c r="D197" s="125">
         <f>SUM(D190:D196)</f>
         <v>1272.73</v>
@@ -34463,11 +34458,11 @@
       <c r="J197" s="129"/>
     </row>
     <row r="198" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A198" s="336" t="s">
+      <c r="A198" s="333" t="s">
         <v>37</v>
       </c>
-      <c r="B198" s="336"/>
-      <c r="C198" s="336"/>
+      <c r="B198" s="333"/>
+      <c r="C198" s="333"/>
       <c r="D198" s="125"/>
       <c r="E198" s="126"/>
       <c r="F198" s="123"/>
@@ -34644,11 +34639,11 @@
       </c>
     </row>
     <row r="204" spans="1:10" ht="18" customHeight="1">
-      <c r="A204" s="336" t="s">
+      <c r="A204" s="333" t="s">
         <v>38</v>
       </c>
-      <c r="B204" s="336"/>
-      <c r="C204" s="336"/>
+      <c r="B204" s="333"/>
+      <c r="C204" s="333"/>
       <c r="D204" s="125">
         <f>SUM(D199:D203)</f>
         <v>786.08</v>
@@ -34666,11 +34661,11 @@
       <c r="J204" s="129"/>
     </row>
     <row r="205" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A205" s="336" t="s">
+      <c r="A205" s="333" t="s">
         <v>38</v>
       </c>
-      <c r="B205" s="336"/>
-      <c r="C205" s="336"/>
+      <c r="B205" s="333"/>
+      <c r="C205" s="333"/>
       <c r="D205" s="125"/>
       <c r="E205" s="126"/>
       <c r="F205" s="123"/>
@@ -34847,11 +34842,11 @@
       </c>
     </row>
     <row r="211" spans="1:10" ht="18" customHeight="1">
-      <c r="A211" s="336" t="s">
+      <c r="A211" s="333" t="s">
         <v>39</v>
       </c>
-      <c r="B211" s="336"/>
-      <c r="C211" s="336"/>
+      <c r="B211" s="333"/>
+      <c r="C211" s="333"/>
       <c r="D211" s="125">
         <f>SUM(D206:D210)</f>
         <v>675.67</v>
@@ -34869,11 +34864,11 @@
       <c r="J211" s="129"/>
     </row>
     <row r="212" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A212" s="336" t="s">
+      <c r="A212" s="333" t="s">
         <v>39</v>
       </c>
-      <c r="B212" s="336"/>
-      <c r="C212" s="336"/>
+      <c r="B212" s="333"/>
+      <c r="C212" s="333"/>
       <c r="D212" s="125"/>
       <c r="E212" s="126"/>
       <c r="F212" s="123"/>
@@ -35050,11 +35045,11 @@
       </c>
     </row>
     <row r="218" spans="1:10" ht="18" customHeight="1">
-      <c r="A218" s="336" t="s">
+      <c r="A218" s="333" t="s">
         <v>40</v>
       </c>
-      <c r="B218" s="336"/>
-      <c r="C218" s="336"/>
+      <c r="B218" s="333"/>
+      <c r="C218" s="333"/>
       <c r="D218" s="125">
         <f>SUM(D213:D217)</f>
         <v>738.56000000000006</v>
@@ -35072,11 +35067,11 @@
       <c r="J218" s="129"/>
     </row>
     <row r="219" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A219" s="336" t="s">
+      <c r="A219" s="333" t="s">
         <v>40</v>
       </c>
-      <c r="B219" s="336"/>
-      <c r="C219" s="336"/>
+      <c r="B219" s="333"/>
+      <c r="C219" s="333"/>
       <c r="D219" s="125"/>
       <c r="E219" s="126"/>
       <c r="F219" s="123"/>
@@ -35189,11 +35184,11 @@
       </c>
     </row>
     <row r="223" spans="1:10" ht="18" customHeight="1">
-      <c r="A223" s="336" t="s">
+      <c r="A223" s="333" t="s">
         <v>41</v>
       </c>
-      <c r="B223" s="336"/>
-      <c r="C223" s="336"/>
+      <c r="B223" s="333"/>
+      <c r="C223" s="333"/>
       <c r="D223" s="125">
         <f>SUM(D220:D222)</f>
         <v>165.10999999999999</v>
@@ -35211,11 +35206,11 @@
       <c r="J223" s="129"/>
     </row>
     <row r="224" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A224" s="336" t="s">
+      <c r="A224" s="333" t="s">
         <v>41</v>
       </c>
-      <c r="B224" s="336"/>
-      <c r="C224" s="336"/>
+      <c r="B224" s="333"/>
+      <c r="C224" s="333"/>
       <c r="D224" s="125"/>
       <c r="E224" s="126"/>
       <c r="F224" s="123"/>
@@ -35360,11 +35355,11 @@
       </c>
     </row>
     <row r="229" spans="1:10" ht="18" customHeight="1">
-      <c r="A229" s="336" t="s">
+      <c r="A229" s="333" t="s">
         <v>42</v>
       </c>
-      <c r="B229" s="336"/>
-      <c r="C229" s="336"/>
+      <c r="B229" s="333"/>
+      <c r="C229" s="333"/>
       <c r="D229" s="125">
         <f>SUM(D225:D228)</f>
         <v>394.7</v>
@@ -35382,11 +35377,11 @@
       <c r="J229" s="129"/>
     </row>
     <row r="230" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A230" s="336" t="s">
+      <c r="A230" s="333" t="s">
         <v>42</v>
       </c>
-      <c r="B230" s="336"/>
-      <c r="C230" s="336"/>
+      <c r="B230" s="333"/>
+      <c r="C230" s="333"/>
       <c r="D230" s="125"/>
       <c r="E230" s="126"/>
       <c r="F230" s="123"/>
@@ -35563,11 +35558,11 @@
       </c>
     </row>
     <row r="236" spans="1:10" ht="18" customHeight="1">
-      <c r="A236" s="336" t="s">
+      <c r="A236" s="333" t="s">
         <v>43</v>
       </c>
-      <c r="B236" s="336"/>
-      <c r="C236" s="336"/>
+      <c r="B236" s="333"/>
+      <c r="C236" s="333"/>
       <c r="D236" s="125">
         <f>SUM(D231:D235)</f>
         <v>642.54999999999995</v>
@@ -35585,11 +35580,11 @@
       <c r="J236" s="129"/>
     </row>
     <row r="237" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A237" s="336" t="s">
+      <c r="A237" s="333" t="s">
         <v>43</v>
       </c>
-      <c r="B237" s="336"/>
-      <c r="C237" s="336"/>
+      <c r="B237" s="333"/>
+      <c r="C237" s="333"/>
       <c r="D237" s="125"/>
       <c r="E237" s="126"/>
       <c r="F237" s="123"/>
@@ -35734,11 +35729,11 @@
       </c>
     </row>
     <row r="242" spans="1:10" ht="18" customHeight="1">
-      <c r="A242" s="336" t="s">
+      <c r="A242" s="333" t="s">
         <v>44</v>
       </c>
-      <c r="B242" s="336"/>
-      <c r="C242" s="336"/>
+      <c r="B242" s="333"/>
+      <c r="C242" s="333"/>
       <c r="D242" s="125">
         <f>SUM(D238:D241)</f>
         <v>603.67000000000007</v>
@@ -35756,11 +35751,11 @@
       <c r="J242" s="129"/>
     </row>
     <row r="243" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A243" s="336" t="s">
+      <c r="A243" s="333" t="s">
         <v>44</v>
       </c>
-      <c r="B243" s="336"/>
-      <c r="C243" s="336"/>
+      <c r="B243" s="333"/>
+      <c r="C243" s="333"/>
       <c r="D243" s="125"/>
       <c r="E243" s="126"/>
       <c r="F243" s="123"/>
@@ -35937,11 +35932,11 @@
       </c>
     </row>
     <row r="249" spans="1:10" ht="18" customHeight="1">
-      <c r="A249" s="336" t="s">
+      <c r="A249" s="333" t="s">
         <v>45</v>
       </c>
-      <c r="B249" s="336"/>
-      <c r="C249" s="336"/>
+      <c r="B249" s="333"/>
+      <c r="C249" s="333"/>
       <c r="D249" s="125">
         <f>SUM(D244:D248)</f>
         <v>259.83999999999997</v>
@@ -35959,11 +35954,11 @@
       <c r="J249" s="129"/>
     </row>
     <row r="250" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A250" s="336" t="s">
+      <c r="A250" s="333" t="s">
         <v>45</v>
       </c>
-      <c r="B250" s="336"/>
-      <c r="C250" s="336"/>
+      <c r="B250" s="333"/>
+      <c r="C250" s="333"/>
       <c r="D250" s="125"/>
       <c r="E250" s="123"/>
       <c r="F250" s="141"/>
@@ -36140,11 +36135,11 @@
       </c>
     </row>
     <row r="256" spans="1:10" ht="18" customHeight="1">
-      <c r="A256" s="336" t="s">
+      <c r="A256" s="333" t="s">
         <v>46</v>
       </c>
-      <c r="B256" s="336"/>
-      <c r="C256" s="336"/>
+      <c r="B256" s="333"/>
+      <c r="C256" s="333"/>
       <c r="D256" s="125">
         <f>SUM(D251:D255)</f>
         <v>1120.8100000000002</v>
@@ -36162,11 +36157,11 @@
       <c r="J256" s="129"/>
     </row>
     <row r="257" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A257" s="336" t="s">
+      <c r="A257" s="333" t="s">
         <v>46</v>
       </c>
-      <c r="B257" s="336"/>
-      <c r="C257" s="336"/>
+      <c r="B257" s="333"/>
+      <c r="C257" s="333"/>
       <c r="D257" s="125"/>
       <c r="E257" s="126"/>
       <c r="F257" s="123"/>
@@ -36311,11 +36306,11 @@
       </c>
     </row>
     <row r="262" spans="1:10" ht="18" customHeight="1">
-      <c r="A262" s="336" t="s">
+      <c r="A262" s="333" t="s">
         <v>47</v>
       </c>
-      <c r="B262" s="336"/>
-      <c r="C262" s="336"/>
+      <c r="B262" s="333"/>
+      <c r="C262" s="333"/>
       <c r="D262" s="125">
         <f>SUM(D258:D261)</f>
         <v>1701.63</v>
@@ -36333,11 +36328,11 @@
       <c r="J262" s="129"/>
     </row>
     <row r="263" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A263" s="336" t="s">
+      <c r="A263" s="333" t="s">
         <v>47</v>
       </c>
-      <c r="B263" s="336"/>
-      <c r="C263" s="336"/>
+      <c r="B263" s="333"/>
+      <c r="C263" s="333"/>
       <c r="D263" s="125"/>
       <c r="E263" s="126"/>
       <c r="F263" s="123"/>
@@ -36482,11 +36477,11 @@
       </c>
     </row>
     <row r="268" spans="1:10" ht="18" customHeight="1">
-      <c r="A268" s="336" t="s">
+      <c r="A268" s="333" t="s">
         <v>48</v>
       </c>
-      <c r="B268" s="336"/>
-      <c r="C268" s="336"/>
+      <c r="B268" s="333"/>
+      <c r="C268" s="333"/>
       <c r="D268" s="144">
         <f>SUM(D264:D267)</f>
         <v>782</v>
@@ -36504,11 +36499,11 @@
       <c r="J268" s="2"/>
     </row>
     <row r="269" spans="1:10" ht="21.9" customHeight="1">
-      <c r="A269" s="336" t="s">
+      <c r="A269" s="333" t="s">
         <v>48</v>
       </c>
-      <c r="B269" s="336"/>
-      <c r="C269" s="336"/>
+      <c r="B269" s="333"/>
+      <c r="C269" s="333"/>
       <c r="D269" s="144"/>
       <c r="E269" s="126"/>
       <c r="F269" s="123"/>
@@ -36525,11 +36520,11 @@
       <c r="J269" s="145"/>
     </row>
     <row r="270" spans="1:10" ht="23.4">
-      <c r="A270" s="315" t="s">
+      <c r="A270" s="312" t="s">
         <v>724</v>
       </c>
-      <c r="B270" s="316"/>
-      <c r="C270" s="317"/>
+      <c r="B270" s="313"/>
+      <c r="C270" s="314"/>
       <c r="D270" s="146"/>
       <c r="E270" s="147"/>
       <c r="F270" s="147"/>
@@ -36546,11 +36541,11 @@
       </c>
     </row>
     <row r="271" spans="1:10" ht="24">
-      <c r="A271" s="315" t="s">
+      <c r="A271" s="312" t="s">
         <v>724</v>
       </c>
-      <c r="B271" s="316"/>
-      <c r="C271" s="317"/>
+      <c r="B271" s="313"/>
+      <c r="C271" s="314"/>
       <c r="D271" s="146"/>
       <c r="E271" s="147"/>
       <c r="F271" s="147"/>
@@ -36567,18 +36562,18 @@
       </c>
     </row>
     <row r="272" spans="1:10" ht="25.2">
-      <c r="A272" s="320" t="s">
+      <c r="A272" s="317" t="s">
         <v>739</v>
       </c>
-      <c r="B272" s="320"/>
-      <c r="C272" s="320"/>
-      <c r="D272" s="320" t="s">
+      <c r="B272" s="317"/>
+      <c r="C272" s="317"/>
+      <c r="D272" s="317" t="s">
         <v>738</v>
       </c>
-      <c r="E272" s="320"/>
-      <c r="F272" s="320"/>
-      <c r="G272" s="320"/>
-      <c r="H272" s="320"/>
+      <c r="E272" s="317"/>
+      <c r="F272" s="317"/>
+      <c r="G272" s="317"/>
+      <c r="H272" s="317"/>
       <c r="I272" s="152">
         <v>100871023</v>
       </c>
@@ -36587,18 +36582,18 @@
       </c>
     </row>
     <row r="273" spans="1:10" ht="46.5" customHeight="1">
-      <c r="A273" s="320" t="s">
+      <c r="A273" s="317" t="s">
         <v>741</v>
       </c>
-      <c r="B273" s="320"/>
-      <c r="C273" s="320"/>
-      <c r="D273" s="333" t="s">
+      <c r="B273" s="317"/>
+      <c r="C273" s="317"/>
+      <c r="D273" s="330" t="s">
         <v>742</v>
       </c>
-      <c r="E273" s="334"/>
-      <c r="F273" s="334"/>
-      <c r="G273" s="334"/>
-      <c r="H273" s="335"/>
+      <c r="E273" s="331"/>
+      <c r="F273" s="331"/>
+      <c r="G273" s="331"/>
+      <c r="H273" s="332"/>
       <c r="I273" s="154">
         <v>194826746</v>
       </c>
@@ -36607,18 +36602,18 @@
       </c>
     </row>
     <row r="274" spans="1:10" ht="25.2">
-      <c r="A274" s="321" t="s">
+      <c r="A274" s="318" t="s">
         <v>740</v>
       </c>
-      <c r="B274" s="322"/>
-      <c r="C274" s="323"/>
-      <c r="D274" s="330" t="s">
+      <c r="B274" s="319"/>
+      <c r="C274" s="320"/>
+      <c r="D274" s="327" t="s">
         <v>743</v>
       </c>
-      <c r="E274" s="331"/>
-      <c r="F274" s="331"/>
-      <c r="G274" s="331"/>
-      <c r="H274" s="332"/>
+      <c r="E274" s="328"/>
+      <c r="F274" s="328"/>
+      <c r="G274" s="328"/>
+      <c r="H274" s="329"/>
       <c r="I274" s="154">
         <v>295697769</v>
       </c>
@@ -36627,16 +36622,16 @@
       </c>
     </row>
     <row r="275" spans="1:10" ht="25.2">
-      <c r="A275" s="324"/>
-      <c r="B275" s="325"/>
-      <c r="C275" s="326"/>
-      <c r="D275" s="330" t="s">
+      <c r="A275" s="321"/>
+      <c r="B275" s="322"/>
+      <c r="C275" s="323"/>
+      <c r="D275" s="327" t="s">
         <v>744</v>
       </c>
-      <c r="E275" s="331"/>
-      <c r="F275" s="331"/>
-      <c r="G275" s="331"/>
-      <c r="H275" s="332"/>
+      <c r="E275" s="328"/>
+      <c r="F275" s="328"/>
+      <c r="G275" s="328"/>
+      <c r="H275" s="329"/>
       <c r="I275" s="154">
         <v>297231546</v>
       </c>
@@ -36645,16 +36640,16 @@
       </c>
     </row>
     <row r="276" spans="1:10" ht="25.2">
-      <c r="A276" s="324"/>
-      <c r="B276" s="325"/>
-      <c r="C276" s="326"/>
-      <c r="D276" s="330" t="s">
+      <c r="A276" s="321"/>
+      <c r="B276" s="322"/>
+      <c r="C276" s="323"/>
+      <c r="D276" s="327" t="s">
         <v>745</v>
       </c>
-      <c r="E276" s="331"/>
-      <c r="F276" s="331"/>
-      <c r="G276" s="331"/>
-      <c r="H276" s="332"/>
+      <c r="E276" s="328"/>
+      <c r="F276" s="328"/>
+      <c r="G276" s="328"/>
+      <c r="H276" s="329"/>
       <c r="I276" s="154">
         <v>1533777</v>
       </c>
@@ -36663,16 +36658,16 @@
       </c>
     </row>
     <row r="277" spans="1:10" ht="25.2">
-      <c r="A277" s="327"/>
-      <c r="B277" s="328"/>
-      <c r="C277" s="329"/>
-      <c r="D277" s="330" t="s">
+      <c r="A277" s="324"/>
+      <c r="B277" s="325"/>
+      <c r="C277" s="326"/>
+      <c r="D277" s="327" t="s">
         <v>743</v>
       </c>
-      <c r="E277" s="331"/>
-      <c r="F277" s="331"/>
-      <c r="G277" s="331"/>
-      <c r="H277" s="332"/>
+      <c r="E277" s="328"/>
+      <c r="F277" s="328"/>
+      <c r="G277" s="328"/>
+      <c r="H277" s="329"/>
       <c r="I277" s="154">
         <v>295697769</v>
       </c>
@@ -36681,25 +36676,25 @@
       </c>
     </row>
     <row r="278" spans="1:10" ht="25.2">
-      <c r="H278" s="318" t="s">
+      <c r="H278" s="315" t="s">
         <v>748</v>
       </c>
-      <c r="I278" s="318"/>
-      <c r="J278" s="318"/>
+      <c r="I278" s="315"/>
+      <c r="J278" s="315"/>
     </row>
     <row r="279" spans="1:10" ht="25.2">
-      <c r="H279" s="319" t="s">
+      <c r="H279" s="316" t="s">
         <v>746</v>
       </c>
-      <c r="I279" s="319"/>
-      <c r="J279" s="319"/>
+      <c r="I279" s="316"/>
+      <c r="J279" s="316"/>
     </row>
     <row r="286" spans="1:10" ht="25.2">
-      <c r="H286" s="319" t="s">
+      <c r="H286" s="316" t="s">
         <v>747</v>
       </c>
-      <c r="I286" s="319"/>
-      <c r="J286" s="319"/>
+      <c r="I286" s="316"/>
+      <c r="J286" s="316"/>
     </row>
   </sheetData>
   <mergeCells count="90">
@@ -36823,41 +36818,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="33.6">
-      <c r="A1" s="337" t="s">
+      <c r="A1" s="334" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="337"/>
-      <c r="C1" s="337"/>
-      <c r="D1" s="337"/>
-      <c r="E1" s="337"/>
-      <c r="F1" s="337"/>
-      <c r="G1" s="337"/>
-      <c r="H1" s="337"/>
-      <c r="I1" s="337"/>
-      <c r="J1" s="337"/>
+      <c r="B1" s="334"/>
+      <c r="C1" s="334"/>
+      <c r="D1" s="334"/>
+      <c r="E1" s="334"/>
+      <c r="F1" s="334"/>
+      <c r="G1" s="334"/>
+      <c r="H1" s="334"/>
+      <c r="I1" s="334"/>
+      <c r="J1" s="334"/>
     </row>
     <row r="2" spans="1:10" ht="33.6">
-      <c r="A2" s="337" t="s">
+      <c r="A2" s="334" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="337"/>
-      <c r="C2" s="337"/>
-      <c r="D2" s="337"/>
-      <c r="E2" s="337"/>
-      <c r="F2" s="337"/>
-      <c r="G2" s="337"/>
-      <c r="H2" s="337"/>
-      <c r="I2" s="337"/>
-      <c r="J2" s="337"/>
+      <c r="B2" s="334"/>
+      <c r="C2" s="334"/>
+      <c r="D2" s="334"/>
+      <c r="E2" s="334"/>
+      <c r="F2" s="334"/>
+      <c r="G2" s="334"/>
+      <c r="H2" s="334"/>
+      <c r="I2" s="334"/>
+      <c r="J2" s="334"/>
     </row>
     <row r="3" spans="1:10" ht="27">
-      <c r="A3" s="358" t="s">
+      <c r="A3" s="355" t="s">
         <v>723</v>
       </c>
-      <c r="B3" s="358"/>
-      <c r="C3" s="358"/>
-      <c r="D3" s="358"/>
-      <c r="E3" s="358"/>
+      <c r="B3" s="355"/>
+      <c r="C3" s="355"/>
+      <c r="D3" s="355"/>
+      <c r="E3" s="355"/>
       <c r="F3" s="120"/>
       <c r="G3" s="120"/>
       <c r="H3" s="120"/>
@@ -36865,12 +36860,12 @@
       <c r="J3" s="120"/>
     </row>
     <row r="4" spans="1:10" ht="27">
-      <c r="A4" s="339" t="s">
+      <c r="A4" s="336" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="339"/>
-      <c r="C4" s="339"/>
-      <c r="D4" s="339"/>
+      <c r="B4" s="336"/>
+      <c r="C4" s="336"/>
+      <c r="D4" s="336"/>
       <c r="E4" s="120"/>
       <c r="F4" s="120"/>
       <c r="G4" s="120"/>
@@ -36879,47 +36874,47 @@
       <c r="J4" s="120"/>
     </row>
     <row r="5" spans="1:10" ht="25.2">
-      <c r="A5" s="359" t="s">
+      <c r="A5" s="356" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="362" t="s">
+      <c r="B5" s="359" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="363"/>
-      <c r="D5" s="364"/>
-      <c r="E5" s="365" t="s">
+      <c r="C5" s="360"/>
+      <c r="D5" s="361"/>
+      <c r="E5" s="362" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="366"/>
-      <c r="G5" s="366"/>
-      <c r="H5" s="366"/>
-      <c r="I5" s="366"/>
-      <c r="J5" s="367" t="s">
+      <c r="F5" s="363"/>
+      <c r="G5" s="363"/>
+      <c r="H5" s="363"/>
+      <c r="I5" s="363"/>
+      <c r="J5" s="364" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="25.2">
-      <c r="A6" s="360"/>
-      <c r="B6" s="370" t="s">
+      <c r="A6" s="357"/>
+      <c r="B6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="371"/>
-      <c r="D6" s="372"/>
-      <c r="E6" s="373" t="s">
+      <c r="C6" s="368"/>
+      <c r="D6" s="369"/>
+      <c r="E6" s="370" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="374" t="s">
+      <c r="F6" s="371" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="370" t="s">
+      <c r="G6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="371"/>
-      <c r="I6" s="372"/>
-      <c r="J6" s="368"/>
+      <c r="H6" s="368"/>
+      <c r="I6" s="369"/>
+      <c r="J6" s="365"/>
     </row>
     <row r="7" spans="1:10" ht="25.2">
-      <c r="A7" s="361"/>
+      <c r="A7" s="358"/>
       <c r="B7" s="155" t="s">
         <v>6</v>
       </c>
@@ -36929,8 +36924,8 @@
       <c r="D7" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="374"/>
-      <c r="F7" s="374"/>
+      <c r="E7" s="371"/>
+      <c r="F7" s="371"/>
       <c r="G7" s="155" t="s">
         <v>6</v>
       </c>
@@ -36940,7 +36935,7 @@
       <c r="I7" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="369"/>
+      <c r="J7" s="366"/>
     </row>
     <row r="8" spans="1:10" ht="18" customHeight="1">
       <c r="A8" s="131">
@@ -37934,10 +37929,10 @@
       <c r="J40" s="156"/>
     </row>
     <row r="41" spans="1:10" ht="24">
-      <c r="A41" s="356" t="s">
+      <c r="A41" s="353" t="s">
         <v>724</v>
       </c>
-      <c r="B41" s="357"/>
+      <c r="B41" s="354"/>
       <c r="C41" s="157"/>
       <c r="D41" s="146">
         <f>SUM(D8:D40)</f>

</xml_diff>